<commit_message>
Find and draft batch 2026-09-28 (19 brands) for Monday send
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_015V3tpdvHrRGbX5pxPwM4Y2
</commit_message>
<xml_diff>
--- a/brands_intl.xlsx
+++ b/brands_intl.xlsx
@@ -423,21 +423,21 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R20"/>
+  <dimension ref="A1:R39"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="16" customWidth="1" min="1" max="1"/>
-    <col width="28" customWidth="1" min="2" max="2"/>
+    <col width="17" customWidth="1" min="1" max="1"/>
+    <col width="36" customWidth="1" min="2" max="2"/>
     <col width="16" customWidth="1" min="3" max="3"/>
     <col width="60" customWidth="1" min="4" max="4"/>
     <col width="12" customWidth="1" min="5" max="5"/>
     <col width="28" customWidth="1" min="6" max="6"/>
     <col width="60" customWidth="1" min="7" max="7"/>
     <col width="18" customWidth="1" min="8" max="8"/>
-    <col width="35" customWidth="1" min="9" max="9"/>
+    <col width="36" customWidth="1" min="9" max="9"/>
     <col width="12" customWidth="1" min="10" max="10"/>
     <col width="60" customWidth="1" min="11" max="11"/>
-    <col width="20" customWidth="1" min="12" max="12"/>
+    <col width="27" customWidth="1" min="12" max="12"/>
     <col width="60" customWidth="1" min="13" max="13"/>
     <col width="60" customWidth="1" min="14" max="14"/>
     <col width="60" customWidth="1" min="15" max="15"/>
@@ -541,22 +541,22 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Ella &amp; Jo</t>
+          <t>My Jolie Candle</t>
         </is>
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>https://ellaandjo.ie/</t>
+          <t>https://myjoliecandle.com/</t>
         </is>
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
-          <t>Ireland</t>
+          <t>France</t>
         </is>
       </c>
       <c r="D2" s="3" t="inlineStr">
         <is>
-          <t>https://ellaandjo.ie/policies/terms-of-service — 'Ella &amp; Jo Cosmetics … Rathglass, Enniscrone, F26 A302, Ireland'</t>
+          <t>https://myjoliecandle.com/pages/mentions-legales — 'siège social … 27520 Grand-Bourgtheroulde, France'</t>
         </is>
       </c>
       <c r="E2" s="2" t="inlineStr">
@@ -566,28 +566,28 @@
       </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t>Beauty / skincare</t>
+          <t>Home / gifts</t>
         </is>
       </c>
       <c r="G2" s="3" t="inlineStr">
         <is>
-          <t>Melt the Day Away Cleansing Balm</t>
+          <t>Bougie bijou My Queen (candle with hidden jewellery)</t>
         </is>
       </c>
       <c r="H2" s="2" t="inlineStr">
         <is>
-          <t>€38</t>
+          <t>€34.90</t>
         </is>
       </c>
       <c r="I2" s="2" t="inlineStr">
         <is>
-          <t>info@ellaandjo.ie</t>
+          <t>partenariats@myjoliecandle.com</t>
         </is>
       </c>
       <c r="J2" s="2" t="inlineStr"/>
       <c r="K2" s="3" t="inlineStr">
         <is>
-          <t>TikTok profile @ellaandjo is a TikTok Shop seller account (ttSeller)</t>
+          <t>TikTok profile @myjoliecandle is a TikTok Shop seller account (ttSeller)</t>
         </is>
       </c>
       <c r="L2" s="2" t="inlineStr">
@@ -597,18 +597,18 @@
       </c>
       <c r="M2" s="3" t="inlineStr">
         <is>
-          <t>none found (checked @ellaandjo bio and @ellaandjo.hu, @ellaandjo.hungary, @ellaandjo.magyarorszag, @ellaandjo_hu, @ellaandjo_hungary, @ellaandjohu, @ellaandjohungary, @ellajo.hu, @ellajo.hungary, @ellajo.magyarorszag, @ellajo_hu, @ellajo_hungary, @ellajohu, @ellajohungary)</t>
+          <t>none found (checked @myjoliecandle bio and @myjoliecandle.hu, @myjoliecandle.hungary, @myjoliecandle.magyarorszag, @myjoliecandle_hu, @myjoliecandle_hungary, @myjoliecandlehu, @myjoliecandlehungary)</t>
         </is>
       </c>
       <c r="N2" s="3" t="inlineStr"/>
       <c r="O2" s="3" t="inlineStr">
         <is>
-          <t>Your Melt the Day Away cleansing balm is easy to demonstrate on camera: makeup on, balm, makeup off, all in one short video.</t>
+          <t>Your jewellery candles, like the My Queen candle, are made for TikTok: the moment the hidden piece of jewellery appears is exactly what keeps people watching a short video.</t>
         </is>
       </c>
       <c r="P2" s="2" t="inlineStr">
         <is>
-          <t>beauty and skincare creators</t>
+          <t>home and lifestyle creators</t>
         </is>
       </c>
       <c r="Q2" s="3" t="inlineStr"/>
@@ -621,12 +621,12 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>SOSU Cosmetics</t>
+          <t>Bare by Vogue</t>
         </is>
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>https://sosucosmetics.com/</t>
+          <t>https://barebyvogue.com/</t>
         </is>
       </c>
       <c r="C3" s="2" t="inlineStr">
@@ -636,7 +636,7 @@
       </c>
       <c r="D3" s="3" t="inlineStr">
         <is>
-          <t>NOT CONFIRMED</t>
+          <t>https://barebyvogue.com/policies/terms-of-service — 'governed by … the laws of Ireland'</t>
         </is>
       </c>
       <c r="E3" s="2" t="inlineStr">
@@ -651,23 +651,23 @@
       </c>
       <c r="G3" s="3" t="inlineStr">
         <is>
-          <t>Dripping Gold Luxury Mousse</t>
-        </is>
-      </c>
-      <c r="H3" s="2" t="inlineStr"/>
+          <t>Overnight Tan Mask</t>
+        </is>
+      </c>
+      <c r="H3" s="2" t="inlineStr">
+        <is>
+          <t>€30</t>
+        </is>
+      </c>
       <c r="I3" s="2" t="inlineStr">
         <is>
-          <t>customerservice@sosucosmetics.com</t>
-        </is>
-      </c>
-      <c r="J3" s="2" t="inlineStr">
-        <is>
-          <t>Suzanne</t>
-        </is>
-      </c>
+          <t>info@barebyvogue.com</t>
+        </is>
+      </c>
+      <c r="J3" s="2" t="inlineStr"/>
       <c r="K3" s="3" t="inlineStr">
         <is>
-          <t>TikTok profile @sosucosmetics is a TikTok Shop seller account (ttSeller)</t>
+          <t>TikTok profile @barebyvogue is a TikTok Shop seller account (ttSeller)</t>
         </is>
       </c>
       <c r="L3" s="2" t="inlineStr">
@@ -677,13 +677,13 @@
       </c>
       <c r="M3" s="3" t="inlineStr">
         <is>
-          <t>none found (checked @sosucosmetics bio and @sosucosmetics.hu, @sosucosmetics.hungary, @sosucosmetics.magyarorszag, @sosucosmetics_hu, @sosucosmetics_hungary, @sosucosmeticshu, @sosucosmeticshungary)</t>
+          <t>none found (checked @barebyvogue bio and @barebyvogue.hu, @barebyvogue.hungary, @barebyvogue.magyarorszag, @barebyvogue_hu, @barebyvogue_hungary, @barebyvoguehu, @barebyvoguehungary)</t>
         </is>
       </c>
       <c r="N3" s="3" t="inlineStr"/>
       <c r="O3" s="3" t="inlineStr">
         <is>
-          <t>Your Dripping Gold Luxury Mousse, marked best seller on your site, is exactly the kind of product that sells on TikTok: the before-and-after is visible in one short video.</t>
+          <t>Your new Overnight Tan Mask is exactly the kind of product that sells on TikTok: apply it at night, show the glow in the morning, all in one short video.</t>
         </is>
       </c>
       <c r="P3" s="2" t="inlineStr">
@@ -691,11 +691,7 @@
           <t>beauty and skincare creators</t>
         </is>
       </c>
-      <c r="Q3" s="3" t="inlineStr">
-        <is>
-          <t>home country not confirmed on the brand's legal/imprint/terms page</t>
-        </is>
-      </c>
+      <c r="Q3" s="3" t="inlineStr"/>
       <c r="R3" s="2" t="inlineStr">
         <is>
           <t>2026-09-26</t>
@@ -705,22 +701,22 @@
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>Claresa</t>
+          <t>Ella &amp; Jo</t>
         </is>
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>https://claresa.pl/</t>
+          <t>https://ellaandjo.ie/</t>
         </is>
       </c>
       <c r="C4" s="2" t="inlineStr">
         <is>
-          <t>Poland</t>
+          <t>Ireland</t>
         </is>
       </c>
       <c r="D4" s="3" t="inlineStr">
         <is>
-          <t>https://claresa.pl/pl/i/Regulamin/3 — '4MASS S.A. … ul. Kobyłkowska 2, 05-200 Wołomin'</t>
+          <t>https://ellaandjo.ie/policies/terms-of-service — 'Ella &amp; Jo Cosmetics … Rathglass, Enniscrone, F26 A302, Ireland'</t>
         </is>
       </c>
       <c r="E4" s="2" t="inlineStr">
@@ -730,28 +726,28 @@
       </c>
       <c r="F4" s="2" t="inlineStr">
         <is>
-          <t>Beauty / nails</t>
+          <t>Beauty / skincare</t>
         </is>
       </c>
       <c r="G4" s="3" t="inlineStr">
         <is>
-          <t>Builder Gel Starter System; hybrid polishes in 300+ colours</t>
+          <t>Melt the Day Away Cleansing Balm</t>
         </is>
       </c>
       <c r="H4" s="2" t="inlineStr">
         <is>
-          <t>130-160 zł</t>
+          <t>€38</t>
         </is>
       </c>
       <c r="I4" s="2" t="inlineStr">
         <is>
-          <t>biuro@claresa.pl</t>
+          <t>info@ellaandjo.ie</t>
         </is>
       </c>
       <c r="J4" s="2" t="inlineStr"/>
       <c r="K4" s="3" t="inlineStr">
         <is>
-          <t>TikTok profile @claresa.pl is a TikTok Shop seller account (ttSeller)</t>
+          <t>TikTok profile @ellaandjo is a TikTok Shop seller account (ttSeller)</t>
         </is>
       </c>
       <c r="L4" s="2" t="inlineStr">
@@ -761,13 +757,13 @@
       </c>
       <c r="M4" s="3" t="inlineStr">
         <is>
-          <t>none found (checked @claresa.pl bio and @claresa.hu, @claresa.hungary, @claresa.magyarorszag, @claresa.pl.hu, @claresa.pl.hungary, @claresa.pl.magyarorszag, @claresa.pl_hu, @claresa.pl_hungary, @claresa.plhu, @claresa.plhungary, @claresa_hu, @claresa_hungary, @claresahu, @claresahungary)</t>
+          <t>none found (checked @ellaandjo bio and @ellaandjo.hu, @ellaandjo.hungary, @ellaandjo.magyarorszag, @ellaandjo_hu, @ellaandjo_hungary, @ellaandjohu, @ellaandjohungary, @ellajo.hu, @ellajo.hungary, @ellajo.magyarorszag, @ellajo_hu, @ellajo_hungary, @ellajohu, @ellajohungary)</t>
         </is>
       </c>
       <c r="N4" s="3" t="inlineStr"/>
       <c r="O4" s="3" t="inlineStr">
         <is>
-          <t>With hybrid polishes in over 300 colours, Claresa is made for nail swatch videos, and your Builder Gel Starter System gives creators a full at-home manicure to film.</t>
+          <t>Your Melt the Day Away cleansing balm is easy to demonstrate on camera: makeup on, balm, makeup off, all in one short video.</t>
         </is>
       </c>
       <c r="P4" s="2" t="inlineStr">
@@ -785,22 +781,22 @@
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>Orientana</t>
+          <t>SOSU Cosmetics</t>
         </is>
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>https://orientana.pl/</t>
+          <t>https://sosucosmetics.com/</t>
         </is>
       </c>
       <c r="C5" s="2" t="inlineStr">
         <is>
-          <t>Poland</t>
+          <t>Ireland</t>
         </is>
       </c>
       <c r="D5" s="3" t="inlineStr">
         <is>
-          <t>https://orientana.pl/pages/regulamin — 'Orientana sp. z o.o. UL. TAMKA 29/17 00-355 WARSZAWA'</t>
+          <t>NOT CONFIRMED</t>
         </is>
       </c>
       <c r="E5" s="2" t="inlineStr">
@@ -810,28 +806,28 @@
       </c>
       <c r="F5" s="2" t="inlineStr">
         <is>
-          <t>Beauty / skincare</t>
+          <t>Beauty / self-tan</t>
         </is>
       </c>
       <c r="G5" s="3" t="inlineStr">
         <is>
-          <t>Sandalwood &amp; turmeric face cream (Krem do twarzy drzewo sandałowe i kurkuma)</t>
-        </is>
-      </c>
-      <c r="H5" s="2" t="inlineStr">
-        <is>
-          <t>55,99 zł</t>
-        </is>
-      </c>
+          <t>Dripping Gold Luxury Mousse</t>
+        </is>
+      </c>
+      <c r="H5" s="2" t="inlineStr"/>
       <c r="I5" s="2" t="inlineStr">
         <is>
-          <t>sklep@orientana.pl</t>
-        </is>
-      </c>
-      <c r="J5" s="2" t="inlineStr"/>
+          <t>customerservice@sosucosmetics.com</t>
+        </is>
+      </c>
+      <c r="J5" s="2" t="inlineStr">
+        <is>
+          <t>Suzanne</t>
+        </is>
+      </c>
       <c r="K5" s="3" t="inlineStr">
         <is>
-          <t>TikTok profile @orientana is a TikTok Shop seller account (ttSeller)</t>
+          <t>TikTok profile @sosucosmetics is a TikTok Shop seller account (ttSeller)</t>
         </is>
       </c>
       <c r="L5" s="2" t="inlineStr">
@@ -841,13 +837,13 @@
       </c>
       <c r="M5" s="3" t="inlineStr">
         <is>
-          <t>none found (checked @orientana bio and @orientana.hu, @orientana.hungary, @orientana.magyarorszag, @orientana_hu, @orientana_hungary, @orientanahu, @orientanahungary)</t>
+          <t>none found (checked @sosucosmetics bio and @sosucosmetics.hu, @sosucosmetics.hungary, @sosucosmetics.magyarorszag, @sosucosmetics_hu, @sosucosmetics_hungary, @sosucosmeticshu, @sosucosmeticshungary)</t>
         </is>
       </c>
       <c r="N5" s="3" t="inlineStr"/>
       <c r="O5" s="3" t="inlineStr">
         <is>
-          <t>Your sandalwood and turmeric face cream, marked as a bestseller on your site, is the kind of product Hungarian creators can show in a simple morning skincare routine video.</t>
+          <t>Your Dripping Gold Luxury Mousse, marked best seller on your site, is exactly the kind of product that sells on TikTok: the before-and-after is visible in one short video.</t>
         </is>
       </c>
       <c r="P5" s="2" t="inlineStr">
@@ -855,7 +851,11 @@
           <t>beauty and skincare creators</t>
         </is>
       </c>
-      <c r="Q5" s="3" t="inlineStr"/>
+      <c r="Q5" s="3" t="inlineStr">
+        <is>
+          <t>home country not confirmed on the brand's legal/imprint/terms page</t>
+        </is>
+      </c>
       <c r="R5" s="2" t="inlineStr">
         <is>
           <t>2026-09-26</t>
@@ -865,12 +865,12 @@
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>PAESE</t>
+          <t>Boska Nails</t>
         </is>
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>https://paese.pl/</t>
+          <t>https://boskanails.pl/</t>
         </is>
       </c>
       <c r="C6" s="2" t="inlineStr">
@@ -880,7 +880,7 @@
       </c>
       <c r="D6" s="3" t="inlineStr">
         <is>
-          <t>https://paese.pl/regulamin/ — 'Euphora Paese Sp. z o.o. ul. Wielicka 28, 30-552 Kraków'</t>
+          <t>https://boskanails.pl/regulaminy — 'BOSKA NAILS SP. Z O.O. z siedzibą … ul. Grzybowska 87' (Warszawa)</t>
         </is>
       </c>
       <c r="E6" s="2" t="inlineStr">
@@ -890,28 +890,28 @@
       </c>
       <c r="F6" s="2" t="inlineStr">
         <is>
-          <t>Beauty / makeup</t>
+          <t>Beauty / nails</t>
         </is>
       </c>
       <c r="G6" s="3" t="inlineStr">
         <is>
-          <t>Puff Cloud ultralight pressed powder with blur effect</t>
+          <t>Base Maestra UV (30 ml)</t>
         </is>
       </c>
       <c r="H6" s="2" t="inlineStr">
         <is>
-          <t>59,90 zł</t>
+          <t>59,99 zł</t>
         </is>
       </c>
       <c r="I6" s="2" t="inlineStr">
         <is>
-          <t>export@paese.pl</t>
+          <t>hello@boskanails.pl</t>
         </is>
       </c>
       <c r="J6" s="2" t="inlineStr"/>
       <c r="K6" s="3" t="inlineStr">
         <is>
-          <t>Site footer links 'Regulamin promocji TikTok Shop'; TikTok profile @paesecosmetics is a TikTok Shop seller account (ttSeller)</t>
+          <t>TikTok profile @boskanailspl is a TikTok Shop seller account (ttSeller)</t>
         </is>
       </c>
       <c r="L6" s="2" t="inlineStr">
@@ -921,13 +921,13 @@
       </c>
       <c r="M6" s="3" t="inlineStr">
         <is>
-          <t>none found (checked @paesecosmetics bio and @paese.hu, @paese.hungary, @paese.magyarorszag, @paese_hu, @paese_hungary, @paesecosmetics.hu, @paesecosmetics.hungary, @paesecosmetics.magyarorszag, @paesecosmetics_hu, @paesecosmetics_hungary, @paesecosmeticshu, @paesecosmeticshungary, @paesehu, @paesehungary)</t>
+          <t>none found (checked @boskanailspl bio and @boskanails.hu, @boskanails.hungary, @boskanails.magyarorszag, @boskanails_hu, @boskanails_hungary, @boskanailshu, @boskanailshungary, @boskanailspl.hu, @boskanailspl.hungary, @boskanailspl.magyarorszag, @boskanailspl_hu, @boskanailspl_hungary, @boskanailsplhu, @boskanailsplhungary)</t>
         </is>
       </c>
       <c r="N6" s="3" t="inlineStr"/>
       <c r="O6" s="3" t="inlineStr">
         <is>
-          <t>Your Puff Cloud pressed powder with a blur effect is exactly the kind of product that sells in a 15-second before-and-after video.</t>
+          <t>Your Base Maestra UV, first in your bestsellers, is easy to show in a short video, from bare nails to a finished manicure on camera.</t>
         </is>
       </c>
       <c r="P6" s="2" t="inlineStr">
@@ -945,12 +945,12 @@
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>Tuban</t>
+          <t>Claresa</t>
         </is>
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
-          <t>https://tuban.pl/</t>
+          <t>https://claresa.pl/</t>
         </is>
       </c>
       <c r="C7" s="2" t="inlineStr">
@@ -960,7 +960,7 @@
       </c>
       <c r="D7" s="3" t="inlineStr">
         <is>
-          <t>https://tuban.pl/regulamin-sklepu/ — 'TUBAN Trade sp. z o.o. ul. Hetmańska 92 43-600 Jaworzno'</t>
+          <t>https://claresa.pl/pl/i/Regulamin/3 — '4MASS S.A. … ul. Kobyłkowska 2, 05-200 Wołomin'</t>
         </is>
       </c>
       <c r="E7" s="2" t="inlineStr">
@@ -970,28 +970,28 @@
       </c>
       <c r="F7" s="2" t="inlineStr">
         <is>
-          <t>Toys / kids</t>
+          <t>Beauty / nails</t>
         </is>
       </c>
       <c r="G7" s="3" t="inlineStr">
         <is>
-          <t>Tubi Jelly Robaki set (Zabawka Roku 2024)</t>
+          <t>Builder Gel Starter System; hybrid polishes in 300+ colours</t>
         </is>
       </c>
       <c r="H7" s="2" t="inlineStr">
         <is>
-          <t>124,74 zł</t>
+          <t>130-160 zł</t>
         </is>
       </c>
       <c r="I7" s="2" t="inlineStr">
         <is>
-          <t>kontakt@tuban.pl</t>
+          <t>biuro@claresa.pl</t>
         </is>
       </c>
       <c r="J7" s="2" t="inlineStr"/>
       <c r="K7" s="3" t="inlineStr">
         <is>
-          <t>TikTok profile @tubantoys is a TikTok Shop seller account (ttSeller)</t>
+          <t>TikTok profile @claresa.pl is a TikTok Shop seller account (ttSeller)</t>
         </is>
       </c>
       <c r="L7" s="2" t="inlineStr">
@@ -1001,22 +1001,18 @@
       </c>
       <c r="M7" s="3" t="inlineStr">
         <is>
-          <t>none found (@tubanhu is an empty namesake: 0 videos, not a seller)</t>
-        </is>
-      </c>
-      <c r="N7" s="3" t="inlineStr">
-        <is>
-          <t>also runs tuban.hu</t>
-        </is>
-      </c>
+          <t>none found (checked @claresa.pl bio and @claresa.hu, @claresa.hungary, @claresa.magyarorszag, @claresa.pl.hu, @claresa.pl.hungary, @claresa.pl.magyarorszag, @claresa.pl_hu, @claresa.pl_hungary, @claresa.plhu, @claresa.plhungary, @claresa_hu, @claresa_hungary, @claresahu, @claresahungary)</t>
+        </is>
+      </c>
+      <c r="N7" s="3" t="inlineStr"/>
       <c r="O7" s="3" t="inlineStr">
         <is>
-          <t>Your Tubi Jelly Robaki set, named Toy of the Year 2024 on your site, is the kind of hands-on toy that sells in a 15-second video: viewers watch the jelly worms being made.</t>
+          <t>With hybrid polishes in over 300 colours, Claresa is made for nail swatch videos, and your Builder Gel Starter System gives creators a full at-home manicure to film.</t>
         </is>
       </c>
       <c r="P7" s="2" t="inlineStr">
         <is>
-          <t>home and lifestyle creators</t>
+          <t>beauty and skincare creators</t>
         </is>
       </c>
       <c r="Q7" s="3" t="inlineStr"/>
@@ -1029,22 +1025,22 @@
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>SINGULARU</t>
+          <t>Noble Health</t>
         </is>
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>https://singularu.com/</t>
+          <t>https://noblehealth.pl/</t>
         </is>
       </c>
       <c r="C8" s="2" t="inlineStr">
         <is>
-          <t>Spain</t>
+          <t>Poland</t>
         </is>
       </c>
       <c r="D8" s="3" t="inlineStr">
         <is>
-          <t>https://singularu.com/pages/aviso-legal — 'SINGULARU IDEAS A MEDIDA, S.L. … España con CIF B-98623937'</t>
+          <t>https://noblehealth.pl/policies/terms-of-service — 'BONATED sp. z o.o. z siedzibą w Warszawie'</t>
         </is>
       </c>
       <c r="E8" s="2" t="inlineStr">
@@ -1054,28 +1050,28 @@
       </c>
       <c r="F8" s="2" t="inlineStr">
         <is>
-          <t>Jewellery</t>
+          <t>Supplements / haircare</t>
         </is>
       </c>
       <c r="G8" s="3" t="inlineStr">
         <is>
-          <t>Collar Chic Pearl (steel, 18kt gold plated)</t>
+          <t>Hair Care Panda Vegan Gummies (biotin)</t>
         </is>
       </c>
       <c r="H8" s="2" t="inlineStr">
         <is>
-          <t>37,99 €</t>
+          <t>105 zł</t>
         </is>
       </c>
       <c r="I8" s="2" t="inlineStr">
         <is>
-          <t>info@singularu.com</t>
+          <t>info@noblehealth.pl</t>
         </is>
       </c>
       <c r="J8" s="2" t="inlineStr"/>
       <c r="K8" s="3" t="inlineStr">
         <is>
-          <t>TikTok profile @singularu is a TikTok Shop seller account (ttSeller)</t>
+          <t>TikTok profile @noble_health is a TikTok Shop seller account (ttSeller)</t>
         </is>
       </c>
       <c r="L8" s="2" t="inlineStr">
@@ -1085,18 +1081,18 @@
       </c>
       <c r="M8" s="3" t="inlineStr">
         <is>
-          <t>none found (checked @singularu bio and @singularu.hu, @singularu.hungary, @singularu.magyarorszag, @singularu_hu, @singularu_hungary, @singularuhu, @singularuhungary)</t>
+          <t>none found (checked @noble_health bio and @noble_health.hu, @noble_health.hungary, @noble_health.magyarorszag, @noble_health_hu, @noble_health_hungary, @noble_healthhu, @noble_healthhungary, @noblehealth.hu, @noblehealth.hungary, @noblehealth.magyarorszag, @noblehealth_hu, @noblehealth_hungary, @noblehealthhu, @noblehealthhungary)</t>
         </is>
       </c>
       <c r="N8" s="3" t="inlineStr"/>
       <c r="O8" s="3" t="inlineStr">
         <is>
-          <t>Your Chic Pearl necklace, which customers can combine with their favourite Singularu charm, is made for short styling videos where creators build a look on camera.</t>
+          <t>Your Hair Care Panda Vegan Gummies, marked Bestseller on your site, are a colourful daily habit that's easy to film, exactly the kind of product that works in a 15-second routine video.</t>
         </is>
       </c>
       <c r="P8" s="2" t="inlineStr">
         <is>
-          <t>fashion and accessories creators</t>
+          <t>beauty and skincare creators</t>
         </is>
       </c>
       <c r="Q8" s="3" t="inlineStr"/>
@@ -1109,22 +1105,22 @@
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>Bellamianta</t>
+          <t>Orientana</t>
         </is>
       </c>
       <c r="B9" s="2" t="inlineStr">
         <is>
-          <t>https://bellamianta.com/</t>
+          <t>https://orientana.pl/</t>
         </is>
       </c>
       <c r="C9" s="2" t="inlineStr">
         <is>
-          <t>United Kingdom</t>
+          <t>Poland</t>
         </is>
       </c>
       <c r="D9" s="3" t="inlineStr">
         <is>
-          <t>https://bellamianta.com/policies/privacy-policy — 'Dungannon Enterprise Centre, 2 Coalisland Rd, Dungannon BT71 6JT' (Northern Ireland)</t>
+          <t>https://orientana.pl/pages/regulamin — 'Orientana sp. z o.o. UL. TAMKA 29/17 00-355 WARSZAWA'</t>
         </is>
       </c>
       <c r="E9" s="2" t="inlineStr">
@@ -1134,28 +1130,28 @@
       </c>
       <c r="F9" s="2" t="inlineStr">
         <is>
-          <t>Beauty / self-tan</t>
+          <t>Beauty / skincare</t>
         </is>
       </c>
       <c r="G9" s="3" t="inlineStr">
         <is>
-          <t>Tanning Mousse</t>
+          <t>Sandalwood &amp; turmeric face cream (Krem do twarzy drzewo sandałowe i kurkuma)</t>
         </is>
       </c>
       <c r="H9" s="2" t="inlineStr">
         <is>
-          <t>£22</t>
+          <t>55,99 zł</t>
         </is>
       </c>
       <c r="I9" s="2" t="inlineStr">
         <is>
-          <t>info@bellamianta.com</t>
+          <t>sklep@orientana.pl</t>
         </is>
       </c>
       <c r="J9" s="2" t="inlineStr"/>
       <c r="K9" s="3" t="inlineStr">
         <is>
-          <t>TikTok profile @bellamianta is a TikTok Shop seller account (ttSeller)</t>
+          <t>TikTok profile @orientana is a TikTok Shop seller account (ttSeller)</t>
         </is>
       </c>
       <c r="L9" s="2" t="inlineStr">
@@ -1165,13 +1161,13 @@
       </c>
       <c r="M9" s="3" t="inlineStr">
         <is>
-          <t>none found (checked @bellamianta bio and @bellamianta.hu, @bellamianta.hungary, @bellamianta.magyarorszag, @bellamianta_hu, @bellamianta_hungary, @bellamiantahu, @bellamiantahungary)</t>
+          <t>none found (checked @orientana bio and @orientana.hu, @orientana.hungary, @orientana.magyarorszag, @orientana_hu, @orientana_hungary, @orientanahu, @orientanahungary)</t>
         </is>
       </c>
       <c r="N9" s="3" t="inlineStr"/>
       <c r="O9" s="3" t="inlineStr">
         <is>
-          <t>Your Tanning Mousse is exactly the kind of product that sells on TikTok: the before-and-after of a self-tan is visible in one short video.</t>
+          <t>Your sandalwood and turmeric face cream, marked as a bestseller on your site, is the kind of product Hungarian creators can show in a simple morning skincare routine video.</t>
         </is>
       </c>
       <c r="P9" s="2" t="inlineStr">
@@ -1189,22 +1185,22 @@
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>Dr Botanicals</t>
+          <t>PAESE</t>
         </is>
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>https://drbotanicals.com/</t>
+          <t>https://paese.pl/</t>
         </is>
       </c>
       <c r="C10" s="2" t="inlineStr">
         <is>
-          <t>United Kingdom</t>
+          <t>Poland</t>
         </is>
       </c>
       <c r="D10" s="3" t="inlineStr">
         <is>
-          <t>https://drbotanicals.com/policies/terms-of-service — 'Dr Botanicals, 8 Holkam Road, Orton Southgate, Peterborough PE2 6TE England'</t>
+          <t>https://paese.pl/regulamin/ — 'Euphora Paese Sp. z o.o. ul. Wielicka 28, 30-552 Kraków'</t>
         </is>
       </c>
       <c r="E10" s="2" t="inlineStr">
@@ -1214,28 +1210,28 @@
       </c>
       <c r="F10" s="2" t="inlineStr">
         <is>
-          <t>Beauty / skincare</t>
+          <t>Beauty / makeup</t>
         </is>
       </c>
       <c r="G10" s="3" t="inlineStr">
         <is>
-          <t>Turmeric Superfood Restoring Treatment Mask 30ml</t>
+          <t>Puff Cloud ultralight pressed powder with blur effect</t>
         </is>
       </c>
       <c r="H10" s="2" t="inlineStr">
         <is>
-          <t>£12.99</t>
+          <t>59,90 zł</t>
         </is>
       </c>
       <c r="I10" s="2" t="inlineStr">
         <is>
-          <t>helpdesk@drbotanicals.com</t>
+          <t>export@paese.pl</t>
         </is>
       </c>
       <c r="J10" s="2" t="inlineStr"/>
       <c r="K10" s="3" t="inlineStr">
         <is>
-          <t>TikTok profile @drbotanicals is a TikTok Shop seller account (ttSeller)</t>
+          <t>Site footer links 'Regulamin promocji TikTok Shop'; TikTok profile @paesecosmetics is a TikTok Shop seller account (ttSeller)</t>
         </is>
       </c>
       <c r="L10" s="2" t="inlineStr">
@@ -1245,13 +1241,13 @@
       </c>
       <c r="M10" s="3" t="inlineStr">
         <is>
-          <t>none found (checked @drbotanicals bio and @drbotanicals.hu, @drbotanicals.hungary, @drbotanicals.magyarorszag, @drbotanicals_hu, @drbotanicals_hungary, @drbotanicalshu, @drbotanicalshungary)</t>
+          <t>none found (checked @paesecosmetics bio and @paese.hu, @paese.hungary, @paese.magyarorszag, @paese_hu, @paese_hungary, @paesecosmetics.hu, @paesecosmetics.hungary, @paesecosmetics.magyarorszag, @paesecosmetics_hu, @paesecosmetics_hungary, @paesecosmeticshu, @paesecosmeticshungary, @paesehu, @paesehungary)</t>
         </is>
       </c>
       <c r="N10" s="3" t="inlineStr"/>
       <c r="O10" s="3" t="inlineStr">
         <is>
-          <t>Your Turmeric Superfood Restoring Treatment Mask, first in your best sellers, is easy to show going on and coming off in a short skincare video.</t>
+          <t>Your Puff Cloud pressed powder with a blur effect is exactly the kind of product that sells in a 15-second before-and-after video.</t>
         </is>
       </c>
       <c r="P10" s="2" t="inlineStr">
@@ -1269,22 +1265,22 @@
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t>Dr.PAWPAW</t>
+          <t>Tuban</t>
         </is>
       </c>
       <c r="B11" s="2" t="inlineStr">
         <is>
-          <t>https://www.drpawpaw.com/</t>
+          <t>https://tuban.pl/</t>
         </is>
       </c>
       <c r="C11" s="2" t="inlineStr">
         <is>
-          <t>United Kingdom</t>
+          <t>Poland</t>
         </is>
       </c>
       <c r="D11" s="3" t="inlineStr">
         <is>
-          <t>https://www.drpawpaw.com/pages/terms-conditions — '4th Floor Devonshire House Elmfield Road, Bromley, BR1 1LT, United Kingdom'</t>
+          <t>https://tuban.pl/regulamin-sklepu/ — 'TUBAN Trade sp. z o.o. ul. Hetmańska 92 43-600 Jaworzno'</t>
         </is>
       </c>
       <c r="E11" s="2" t="inlineStr">
@@ -1294,28 +1290,28 @@
       </c>
       <c r="F11" s="2" t="inlineStr">
         <is>
-          <t>Beauty / lip care</t>
+          <t>Toys / kids</t>
         </is>
       </c>
       <c r="G11" s="3" t="inlineStr">
         <is>
-          <t>Scented Charm Balm Trio Pack (banana, matcha, cherry)</t>
+          <t>Tubi Jelly Robaki set (Zabawka Roku 2024)</t>
         </is>
       </c>
       <c r="H11" s="2" t="inlineStr">
         <is>
-          <t>£10.99</t>
+          <t>124,74 zł</t>
         </is>
       </c>
       <c r="I11" s="2" t="inlineStr">
         <is>
-          <t>info@drpawpaw.com</t>
+          <t>kontakt@tuban.pl</t>
         </is>
       </c>
       <c r="J11" s="2" t="inlineStr"/>
       <c r="K11" s="3" t="inlineStr">
         <is>
-          <t>TikTok profile @dr.pawpaw is a TikTok Shop seller account (ttSeller)</t>
+          <t>TikTok profile @tubantoys is a TikTok Shop seller account (ttSeller)</t>
         </is>
       </c>
       <c r="L11" s="2" t="inlineStr">
@@ -1325,18 +1321,22 @@
       </c>
       <c r="M11" s="3" t="inlineStr">
         <is>
-          <t>none found (checked @dr.pawpaw bio and @dr.pawpaw.hu, @dr.pawpaw.hungary, @dr.pawpaw.magyarorszag, @dr.pawpaw_hu, @dr.pawpaw_hungary, @dr.pawpawhu, @dr.pawpawhungary, @drpawpaw.hu, @drpawpaw.hungary, @drpawpaw.magyarorszag, @drpawpaw_hu, @drpawpaw_hungary, @drpawpawhu, @drpawpawhungary)</t>
-        </is>
-      </c>
-      <c r="N11" s="3" t="inlineStr"/>
+          <t>none found (@tubanhu is an empty namesake: 0 videos, not a seller)</t>
+        </is>
+      </c>
+      <c r="N11" s="3" t="inlineStr">
+        <is>
+          <t>also runs tuban.hu</t>
+        </is>
+      </c>
       <c r="O11" s="3" t="inlineStr">
         <is>
-          <t>Your Charm Balm Trio in banana, matcha and cherry is a colourful, giftable set that's easy to show in a short unboxing video.</t>
+          <t>Your Tubi Jelly Robaki set, named Toy of the Year 2024 on your site, is the kind of hands-on toy that sells in a 15-second video: viewers watch the jelly worms being made.</t>
         </is>
       </c>
       <c r="P11" s="2" t="inlineStr">
         <is>
-          <t>beauty and skincare creators</t>
+          <t>home and lifestyle creators</t>
         </is>
       </c>
       <c r="Q11" s="3" t="inlineStr"/>
@@ -1349,22 +1349,22 @@
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>Fable &amp; Mane</t>
+          <t>SINGULARU</t>
         </is>
       </c>
       <c r="B12" s="2" t="inlineStr">
         <is>
-          <t>https://fableandmane.com/</t>
+          <t>https://singularu.com/</t>
         </is>
       </c>
       <c r="C12" s="2" t="inlineStr">
         <is>
-          <t>United Kingdom</t>
+          <t>Spain</t>
         </is>
       </c>
       <c r="D12" s="3" t="inlineStr">
         <is>
-          <t>https://fableandmane.com/policies/terms-of-service — 'write to us at: 30-31 Plympton Street, London, NW8 8AB'</t>
+          <t>https://singularu.com/pages/aviso-legal — 'SINGULARU IDEAS A MEDIDA, S.L. … España con CIF B-98623937'</t>
         </is>
       </c>
       <c r="E12" s="2" t="inlineStr">
@@ -1374,28 +1374,28 @@
       </c>
       <c r="F12" s="2" t="inlineStr">
         <is>
-          <t>Beauty / haircare</t>
+          <t>Jewellery</t>
         </is>
       </c>
       <c r="G12" s="3" t="inlineStr">
         <is>
-          <t>HoliRoots Pre-Wash Scalp &amp; Hair Oil</t>
+          <t>Collar Chic Pearl (steel, 18kt gold plated)</t>
         </is>
       </c>
       <c r="H12" s="2" t="inlineStr">
         <is>
-          <t>$38 / £34</t>
+          <t>37,99 €</t>
         </is>
       </c>
       <c r="I12" s="2" t="inlineStr">
         <is>
-          <t>support@fableandmane.com</t>
+          <t>info@singularu.com</t>
         </is>
       </c>
       <c r="J12" s="2" t="inlineStr"/>
       <c r="K12" s="3" t="inlineStr">
         <is>
-          <t>TikTok profile @fableandmane is a TikTok Shop seller account (ttSeller)</t>
+          <t>TikTok profile @singularu is a TikTok Shop seller account (ttSeller)</t>
         </is>
       </c>
       <c r="L12" s="2" t="inlineStr">
@@ -1405,18 +1405,18 @@
       </c>
       <c r="M12" s="3" t="inlineStr">
         <is>
-          <t>none found (checked @fableandmane bio and @fableandmane.hu, @fableandmane.hungary, @fableandmane.magyarorszag, @fableandmane_hu, @fableandmane_hungary, @fableandmanehu, @fableandmanehungary, @fablemane.hu, @fablemane.hungary, @fablemane.magyarorszag, @fablemane_hu, @fablemane_hungary, @fablemanehu, @fablemanehungary)</t>
+          <t>none found (checked @singularu bio and @singularu.hu, @singularu.hungary, @singularu.magyarorszag, @singularu_hu, @singularu_hungary, @singularuhu, @singularuhungary)</t>
         </is>
       </c>
       <c r="N12" s="3" t="inlineStr"/>
       <c r="O12" s="3" t="inlineStr">
         <is>
-          <t>Your HoliRoots pre-wash scalp and hair oil is an easy product to demonstrate in a short wash-day routine video.</t>
+          <t>Your Chic Pearl necklace, which customers can combine with their favourite Singularu charm, is made for short styling videos where creators build a look on camera.</t>
         </is>
       </c>
       <c r="P12" s="2" t="inlineStr">
         <is>
-          <t>beauty and skincare creators</t>
+          <t>fashion and accessories creators</t>
         </is>
       </c>
       <c r="Q12" s="3" t="inlineStr"/>
@@ -1429,12 +1429,12 @@
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
         <is>
-          <t>Glow Hub</t>
+          <t>Beauty Kitchen</t>
         </is>
       </c>
       <c r="B13" s="2" t="inlineStr">
         <is>
-          <t>https://glowhub.com/</t>
+          <t>https://beautykitchen.co.uk/</t>
         </is>
       </c>
       <c r="C13" s="2" t="inlineStr">
@@ -1444,7 +1444,7 @@
       </c>
       <c r="D13" s="3" t="inlineStr">
         <is>
-          <t>https://glowhub.com/pages/terms-conditions — 'registered in England and Wales … Knutsford, Cheshire, WA16 8ZR' (Amelia Knight Ltd)</t>
+          <t>https://beautykitchen.co.uk/pages/terms-conditions — 'registered address is 121 Netherton Street, Wishaw, ML2 0EF, Company Number SC476415'</t>
         </is>
       </c>
       <c r="E13" s="2" t="inlineStr">
@@ -1454,28 +1454,28 @@
       </c>
       <c r="F13" s="2" t="inlineStr">
         <is>
-          <t>Beauty / skincare &amp; makeup</t>
+          <t>Beauty / skincare</t>
         </is>
       </c>
       <c r="G13" s="3" t="inlineStr">
         <is>
-          <t>BABY BEAM dew filter glow base</t>
+          <t>Seahorse Plankton+ Really Radiant Moisturiser 60ml</t>
         </is>
       </c>
       <c r="H13" s="2" t="inlineStr">
         <is>
-          <t>£11.20</t>
+          <t>£24.50</t>
         </is>
       </c>
       <c r="I13" s="2" t="inlineStr">
         <is>
-          <t>hello@glowhub.com</t>
+          <t>hello@beautykitchen.co.uk</t>
         </is>
       </c>
       <c r="J13" s="2" t="inlineStr"/>
       <c r="K13" s="3" t="inlineStr">
         <is>
-          <t>Site T&amp;Cs mention 'Glow Hub's TikTok shop'; TikTok profile @glowhubbeauty is a TikTok Shop seller account (ttSeller)</t>
+          <t>TikTok profile @beautykitchentiktok is a TikTok Shop seller account (ttSeller)</t>
         </is>
       </c>
       <c r="L13" s="2" t="inlineStr">
@@ -1485,13 +1485,13 @@
       </c>
       <c r="M13" s="3" t="inlineStr">
         <is>
-          <t>none found (checked @glowhubbeauty bio and @glowhub.hu, @glowhub.hungary, @glowhub.magyarorszag, @glowhub_hu, @glowhub_hungary, @glowhubbeauty.hu, @glowhubbeauty.hungary, @glowhubbeauty.magyarorszag, @glowhubbeauty_hu, @glowhubbeauty_hungary, @glowhubbeautyhu, @glowhubbeautyhungary, @glowhubhu, @glowhubhungary)</t>
+          <t>none found (checked @beautykitchentiktok bio and @beautykitchen.hu, @beautykitchen.hungary, @beautykitchen.magyarorszag, @beautykitchen_hu, @beautykitchen_hungary, @beautykitchenhu, @beautykitchenhungary, @beautykitchentiktok.hu, @beautykitchentiktok.hungary, @beautykitchentiktok.magyarorszag, @beautykitchentiktok_hu, @beautykitchentiktok_hungary, @beautykitchentiktokhu, @beautykitchentiktokhungary)</t>
         </is>
       </c>
       <c r="N13" s="3" t="inlineStr"/>
       <c r="O13" s="3" t="inlineStr">
         <is>
-          <t>Your BABY BEAM dew filter glow base is exactly the kind of product that sells in a 15-second before-and-after video, because a dewy finish is easy to show on camera.</t>
+          <t>Your Seahorse Plankton+ Really Radiant Moisturiser has a name and story creators can explain in seconds, which is what makes a skincare product work in a short video.</t>
         </is>
       </c>
       <c r="P13" s="2" t="inlineStr">
@@ -1509,12 +1509,12 @@
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>Hairburst</t>
+          <t>Bellamianta</t>
         </is>
       </c>
       <c r="B14" s="2" t="inlineStr">
         <is>
-          <t>https://www.hairburst.com/</t>
+          <t>https://bellamianta.com/</t>
         </is>
       </c>
       <c r="C14" s="2" t="inlineStr">
@@ -1524,7 +1524,7 @@
       </c>
       <c r="D14" s="3" t="inlineStr">
         <is>
-          <t>https://www.hairburst.com/pages/terms-of-service — 'Registered in England with company number 08898301'</t>
+          <t>https://bellamianta.com/policies/privacy-policy — 'Dungannon Enterprise Centre, 2 Coalisland Rd, Dungannon BT71 6JT' (Northern Ireland)</t>
         </is>
       </c>
       <c r="E14" s="2" t="inlineStr">
@@ -1534,28 +1534,28 @@
       </c>
       <c r="F14" s="2" t="inlineStr">
         <is>
-          <t>Beauty / haircare</t>
+          <t>Beauty / self-tan</t>
         </is>
       </c>
       <c r="G14" s="3" t="inlineStr">
         <is>
-          <t>Chewable Hair Vitamins (hair gummies)</t>
+          <t>Tanning Mousse</t>
         </is>
       </c>
       <c r="H14" s="2" t="inlineStr">
         <is>
-          <t>£22.99 (1 month)</t>
+          <t>£22</t>
         </is>
       </c>
       <c r="I14" s="2" t="inlineStr">
         <is>
-          <t>support@hairburst.com</t>
+          <t>info@bellamianta.com</t>
         </is>
       </c>
       <c r="J14" s="2" t="inlineStr"/>
       <c r="K14" s="3" t="inlineStr">
         <is>
-          <t>TikTok profile @hairburst is a TikTok Shop seller account (ttSeller)</t>
+          <t>TikTok profile @bellamianta is a TikTok Shop seller account (ttSeller)</t>
         </is>
       </c>
       <c r="L14" s="2" t="inlineStr">
@@ -1565,17 +1565,13 @@
       </c>
       <c r="M14" s="3" t="inlineStr">
         <is>
-          <t>none found (checked @hairburst bio and @hairburst.hu, @hairburst.hungary, @hairburst.magyarorszag, @hairburst_hu, @hairburst_hungary, @hairbursthu, @hairbursthungary)</t>
-        </is>
-      </c>
-      <c r="N14" s="3" t="inlineStr">
-        <is>
-          <t>Hungarian site version hairburst.com/hu-hu</t>
-        </is>
-      </c>
+          <t>none found (checked @bellamianta bio and @bellamianta.hu, @bellamianta.hungary, @bellamianta.magyarorszag, @bellamianta_hu, @bellamianta_hungary, @bellamiantahu, @bellamiantahungary)</t>
+        </is>
+      </c>
+      <c r="N14" s="3" t="inlineStr"/>
       <c r="O14" s="3" t="inlineStr">
         <is>
-          <t>Your chewable hair vitamins are an easy daily habit to film, and a hair routine gives creators a natural reason to post updates over several weeks.</t>
+          <t>Your Tanning Mousse is exactly the kind of product that sells on TikTok: the before-and-after of a self-tan is visible in one short video.</t>
         </is>
       </c>
       <c r="P14" s="2" t="inlineStr">
@@ -1593,12 +1589,12 @@
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
         <is>
-          <t>Nala's Baby</t>
+          <t>BetterYou</t>
         </is>
       </c>
       <c r="B15" s="2" t="inlineStr">
         <is>
-          <t>https://nalasbaby.com/</t>
+          <t>https://betteryou.com/</t>
         </is>
       </c>
       <c r="C15" s="2" t="inlineStr">
@@ -1608,7 +1604,7 @@
       </c>
       <c r="D15" s="3" t="inlineStr">
         <is>
-          <t>https://nalasbaby.com/pages/terms-conditions — 'governed by … the laws of England and Wales'</t>
+          <t>https://betteryou.com/pages/terms-conditions — '… Barnsley England S74 9LH Registered Company No: 05541287'</t>
         </is>
       </c>
       <c r="E15" s="2" t="inlineStr">
@@ -1618,28 +1614,28 @@
       </c>
       <c r="F15" s="2" t="inlineStr">
         <is>
-          <t>Baby / kids care</t>
+          <t>Supplements / wellness</t>
         </is>
       </c>
       <c r="G15" s="3" t="inlineStr">
         <is>
-          <t>Nala's Baby Bath-time Gift Set</t>
+          <t>Magnesium Max 3-in-1 Original Powder</t>
         </is>
       </c>
       <c r="H15" s="2" t="inlineStr">
         <is>
-          <t>£25.99</t>
+          <t>£9.99</t>
         </is>
       </c>
       <c r="I15" s="2" t="inlineStr">
         <is>
-          <t>info@nalasbaby.com</t>
+          <t>wecare@betteryou.com</t>
         </is>
       </c>
       <c r="J15" s="2" t="inlineStr"/>
       <c r="K15" s="3" t="inlineStr">
         <is>
-          <t>TikTok profile @nalasbaby is a TikTok Shop seller account (ttSeller) named "Nala's Baby UK"</t>
+          <t>TikTok profile @betteryou_ltd is a TikTok Shop seller account (ttSeller)</t>
         </is>
       </c>
       <c r="L15" s="2" t="inlineStr">
@@ -1649,18 +1645,18 @@
       </c>
       <c r="M15" s="3" t="inlineStr">
         <is>
-          <t>none found (checked @nalasbaby bio and @nalasbaby.hu, @nalasbaby.hungary, @nalasbaby.magyarorszag, @nalasbaby_hu, @nalasbaby_hungary, @nalasbabyhu, @nalasbabyhungary)</t>
+          <t>none found (checked @betteryou_ltd bio and @betteryou.hu, @betteryou.hungary, @betteryou.magyarorszag, @betteryou_hu, @betteryou_hungary, @betteryou_ltd.hu, @betteryou_ltd.hungary, @betteryou_ltd.magyarorszag, @betteryou_ltd_hu, @betteryou_ltd_hungary, @betteryou_ltdhu, @betteryou_ltdhungary, @betteryouhu, @betteryouhungary)</t>
         </is>
       </c>
       <c r="N15" s="3" t="inlineStr"/>
       <c r="O15" s="3" t="inlineStr">
         <is>
-          <t>Your Bath-time Gift Set is a ready-made, giftable bundle, and bath time is one of the easiest family moments to show in a short video.</t>
+          <t>Your Magnesium Max 3-in-1 powder, marked Bestseller on your site, is easy to show in a short video: a scoop, a stir and a daily routine creators can film in seconds.</t>
         </is>
       </c>
       <c r="P15" s="2" t="inlineStr">
         <is>
-          <t>home and lifestyle creators</t>
+          <t>fitness creators</t>
         </is>
       </c>
       <c r="Q15" s="3" t="inlineStr"/>
@@ -1673,12 +1669,12 @@
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t>Novomins</t>
+          <t>BPerfect</t>
         </is>
       </c>
       <c r="B16" s="2" t="inlineStr">
         <is>
-          <t>https://novomins.com/</t>
+          <t>https://www.bperfectcosmetics.com/</t>
         </is>
       </c>
       <c r="C16" s="2" t="inlineStr">
@@ -1688,7 +1684,7 @@
       </c>
       <c r="D16" s="3" t="inlineStr">
         <is>
-          <t>https://novomins.com/policies/terms-of-service — 'operated by Innocent Health Ltd … laws of England and Wales'</t>
+          <t>https://www.bperfectcosmetics.com/policies/terms-of-service — 'registered office is: Block E, Knockmore Industrial Estate, Moira Road, Lisburn. BT28 2EJ' (Northern Ireland)</t>
         </is>
       </c>
       <c r="E16" s="2" t="inlineStr">
@@ -1698,44 +1694,44 @@
       </c>
       <c r="F16" s="2" t="inlineStr">
         <is>
-          <t>Supplements / beauty</t>
+          <t>Beauty / makeup &amp; tan</t>
         </is>
       </c>
       <c r="G16" s="3" t="inlineStr">
         <is>
-          <t>Collagen Gummies (Best Seller)</t>
+          <t>Mrs Glam - Instant Bronze Boost Gel Drops</t>
         </is>
       </c>
       <c r="H16" s="2" t="inlineStr">
         <is>
-          <t>£19.99</t>
+          <t>£16.95</t>
         </is>
       </c>
       <c r="I16" s="2" t="inlineStr">
         <is>
-          <t>hello@novomins.com</t>
+          <t>customercare@bperfectcosmetics.com</t>
         </is>
       </c>
       <c r="J16" s="2" t="inlineStr"/>
       <c r="K16" s="3" t="inlineStr">
         <is>
-          <t>TikTok profile @novominsnutrition is a TikTok Shop seller account (ttSeller)</t>
+          <t>About page: 'one of the Top 3 UK brands on TikTok Shop'; TikTok profile @bperfectcosmetics is a TikTok Shop seller account (ttSeller)</t>
         </is>
       </c>
       <c r="L16" s="2" t="inlineStr">
         <is>
-          <t>not confirmed</t>
+          <t>UK (confirmed: from site)</t>
         </is>
       </c>
       <c r="M16" s="3" t="inlineStr">
         <is>
-          <t>none found (checked @novominsnutrition bio and @novomins.hu, @novomins.hungary, @novomins.magyarorszag, @novomins_hu, @novomins_hungary, @novominshu, @novominshungary, @novominsnutrition.hu, @novominsnutrition.hungary, @novominsnutrition.magyarorszag, @novominsnutrition_hu, @novominsnutrition_hungary, @novominsnutritionhu, @novominsnutritionhungary)</t>
+          <t>none found (checked @bperfectcosmetics bio and @bperfect.hu, @bperfect.hungary, @bperfect.magyarorszag, @bperfect_hu, @bperfect_hungary, @bperfectcosmetics.hu, @bperfectcosmetics.hungary, @bperfectcosmetics.magyarorszag, @bperfectcosmetics_hu, @bperfectcosmetics_hungary, @bperfectcosmeticshu, @bperfectcosmeticshungary, @bperfecthu, @bperfecthungary)</t>
         </is>
       </c>
       <c r="N16" s="3" t="inlineStr"/>
       <c r="O16" s="3" t="inlineStr">
         <is>
-          <t>Your Collagen Gummies, marked Best Seller on your site, are an easy daily habit to film, and gummies are far more fun on camera than a capsule.</t>
+          <t>Your Mrs Glam Instant Bronze Boost Gel Drops are exactly the kind of product that sells in a 15-second before-and-after video.</t>
         </is>
       </c>
       <c r="P16" s="2" t="inlineStr">
@@ -1753,12 +1749,12 @@
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
         <is>
-          <t>Tangle Angel</t>
+          <t>BYBI</t>
         </is>
       </c>
       <c r="B17" s="2" t="inlineStr">
         <is>
-          <t>https://tangleangel.com/</t>
+          <t>https://bybi.com/</t>
         </is>
       </c>
       <c r="C17" s="2" t="inlineStr">
@@ -1768,7 +1764,7 @@
       </c>
       <c r="D17" s="3" t="inlineStr">
         <is>
-          <t>https://tangleangel.com/policies/terms-of-service — 'Tangle Angel Limited, Registered in England … 1 Duchess Street, London W1W 6AN'</t>
+          <t>https://bybi.com/policies/terms-of-service — 'Mystic Elements Limited, a company registered in England and Wales … trading as BYBI'</t>
         </is>
       </c>
       <c r="E17" s="2" t="inlineStr">
@@ -1778,28 +1774,28 @@
       </c>
       <c r="F17" s="2" t="inlineStr">
         <is>
-          <t>Beauty / hair tools</t>
+          <t>Beauty / skincare</t>
         </is>
       </c>
       <c r="G17" s="3" t="inlineStr">
         <is>
-          <t>ANGEL 2.0 detangling brush</t>
+          <t>Strawberry Booster</t>
         </is>
       </c>
       <c r="H17" s="2" t="inlineStr">
         <is>
-          <t>£15</t>
+          <t>£22</t>
         </is>
       </c>
       <c r="I17" s="2" t="inlineStr">
         <is>
-          <t>info@tangleangel.com</t>
+          <t>hey@bybi.com</t>
         </is>
       </c>
       <c r="J17" s="2" t="inlineStr"/>
       <c r="K17" s="3" t="inlineStr">
         <is>
-          <t>TikTok profile @tangleangel is a TikTok Shop seller account (ttSeller)</t>
+          <t>TikTok profile @bybibeauty is a TikTok Shop seller account (ttSeller)</t>
         </is>
       </c>
       <c r="L17" s="2" t="inlineStr">
@@ -1809,13 +1805,13 @@
       </c>
       <c r="M17" s="3" t="inlineStr">
         <is>
-          <t>none found (checked @tangleangel bio and @tangleangel.hu, @tangleangel.hungary, @tangleangel.magyarorszag, @tangleangel_hu, @tangleangel_hungary, @tangleangelhu, @tangleangelhungary)</t>
+          <t>none found (checked @bybibeauty bio and @bybi.hu, @bybi.hungary, @bybi.magyarorszag, @bybi_hu, @bybi_hungary, @bybibeauty.hu, @bybibeauty.hungary, @bybibeauty.magyarorszag, @bybibeauty_hu, @bybibeauty_hungary, @bybibeautyhu, @bybibeautyhungary, @bybihu, @bybihungary)</t>
         </is>
       </c>
       <c r="N17" s="3" t="inlineStr"/>
       <c r="O17" s="3" t="inlineStr">
         <is>
-          <t>Your ANGEL 2.0 detangling brush is exactly the kind of product that sells in a 15-second demo video: one pass through knotted hair shows the result.</t>
+          <t>Your Strawberry Booster, part of your new BYBI Drops, is easy to show in a 15-second skincare routine video.</t>
         </is>
       </c>
       <c r="P17" s="2" t="inlineStr">
@@ -1833,65 +1829,77 @@
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
         <is>
-          <t>Clochee</t>
+          <t>Dr Botanicals</t>
         </is>
       </c>
       <c r="B18" s="2" t="inlineStr">
         <is>
-          <t>https://www.clochee.com/</t>
+          <t>https://drbotanicals.com/</t>
         </is>
       </c>
       <c r="C18" s="2" t="inlineStr">
         <is>
-          <t>Poland</t>
+          <t>United Kingdom</t>
         </is>
       </c>
       <c r="D18" s="3" t="inlineStr">
         <is>
-          <t>https://www.clochee.com/en/terms — 'Clochee Sp. z o o … Szczecin (POLAND)'</t>
+          <t>https://drbotanicals.com/policies/terms-of-service — 'Dr Botanicals, 8 Holkam Road, Orton Southgate, Peterborough PE2 6TE England'</t>
         </is>
       </c>
       <c r="E18" s="2" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>A</t>
         </is>
       </c>
       <c r="F18" s="2" t="inlineStr">
         <is>
-          <t>Natural cosmetics</t>
-        </is>
-      </c>
-      <c r="G18" s="3" t="inlineStr"/>
-      <c r="H18" s="2" t="inlineStr"/>
+          <t>Beauty / skincare</t>
+        </is>
+      </c>
+      <c r="G18" s="3" t="inlineStr">
+        <is>
+          <t>Turmeric Superfood Restoring Treatment Mask 30ml</t>
+        </is>
+      </c>
+      <c r="H18" s="2" t="inlineStr">
+        <is>
+          <t>£12.99</t>
+        </is>
+      </c>
       <c r="I18" s="2" t="inlineStr">
         <is>
-          <t>sklep@clochee.com</t>
+          <t>helpdesk@drbotanicals.com</t>
         </is>
       </c>
       <c r="J18" s="2" t="inlineStr"/>
       <c r="K18" s="3" t="inlineStr">
         <is>
-          <t>none on site; TikTok profile not a seller account</t>
-        </is>
-      </c>
-      <c r="L18" s="2" t="inlineStr"/>
-      <c r="M18" s="3" t="inlineStr"/>
-      <c r="N18" s="3" t="inlineStr">
-        <is>
-          <t>Hungary (Węgry) in shipping country selector</t>
-        </is>
-      </c>
-      <c r="O18" s="3" t="inlineStr"/>
+          <t>TikTok profile @drbotanicals is a TikTok Shop seller account (ttSeller)</t>
+        </is>
+      </c>
+      <c r="L18" s="2" t="inlineStr">
+        <is>
+          <t>not confirmed</t>
+        </is>
+      </c>
+      <c r="M18" s="3" t="inlineStr">
+        <is>
+          <t>none found (checked @drbotanicals bio and @drbotanicals.hu, @drbotanicals.hungary, @drbotanicals.magyarorszag, @drbotanicals_hu, @drbotanicals_hungary, @drbotanicalshu, @drbotanicalshungary)</t>
+        </is>
+      </c>
+      <c r="N18" s="3" t="inlineStr"/>
+      <c r="O18" s="3" t="inlineStr">
+        <is>
+          <t>Your Turmeric Superfood Restoring Treatment Mask, first in your best sellers, is easy to show going on and coming off in a short skincare video.</t>
+        </is>
+      </c>
       <c r="P18" s="2" t="inlineStr">
         <is>
           <t>beauty and skincare creators</t>
         </is>
       </c>
-      <c r="Q18" s="3" t="inlineStr">
-        <is>
-          <t>no specific opener found on site; no featured product; no specific featured product found on site</t>
-        </is>
-      </c>
+      <c r="Q18" s="3" t="inlineStr"/>
       <c r="R18" s="2" t="inlineStr">
         <is>
           <t>2026-09-26</t>
@@ -1901,65 +1909,69 @@
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
         <is>
-          <t>Mokosh</t>
+          <t>Dr.PAWPAW</t>
         </is>
       </c>
       <c r="B19" s="2" t="inlineStr">
         <is>
-          <t>https://mokosh.pl/</t>
+          <t>https://www.drpawpaw.com/</t>
         </is>
       </c>
       <c r="C19" s="2" t="inlineStr">
         <is>
-          <t>Poland</t>
+          <t>United Kingdom</t>
         </is>
       </c>
       <c r="D19" s="3" t="inlineStr">
         <is>
-          <t>https://mokosh.pl/policies/terms-of-service — 'MOKOSH Didiuk sp. k. z siedzibą: ul. Dolna 14, 05-152 Kazuń Nowy'</t>
+          <t>https://www.drpawpaw.com/pages/terms-conditions — '4th Floor Devonshire House Elmfield Road, Bromley, BR1 1LT, United Kingdom'</t>
         </is>
       </c>
       <c r="E19" s="2" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>A</t>
         </is>
       </c>
       <c r="F19" s="2" t="inlineStr">
         <is>
-          <t>Beauty / natural cosmetics</t>
+          <t>Beauty / lip care</t>
         </is>
       </c>
       <c r="G19" s="3" t="inlineStr">
         <is>
-          <t>Bronzing body &amp; face balm, orange with cinnamon</t>
+          <t>Scented Charm Balm Trio Pack (banana, matcha, cherry)</t>
         </is>
       </c>
       <c r="H19" s="2" t="inlineStr">
         <is>
-          <t>89 zł</t>
+          <t>£10.99</t>
         </is>
       </c>
       <c r="I19" s="2" t="inlineStr">
         <is>
-          <t>biuro@mokosh.pl</t>
+          <t>info@drpawpaw.com</t>
         </is>
       </c>
       <c r="J19" s="2" t="inlineStr"/>
       <c r="K19" s="3" t="inlineStr">
         <is>
-          <t>none on site; TikTok profile not a seller account</t>
-        </is>
-      </c>
-      <c r="L19" s="2" t="inlineStr"/>
-      <c r="M19" s="3" t="inlineStr"/>
-      <c r="N19" s="3" t="inlineStr">
-        <is>
-          <t>Site lists Hungary (Węgry) among countries where Mokosh sells</t>
-        </is>
-      </c>
+          <t>TikTok profile @dr.pawpaw is a TikTok Shop seller account (ttSeller)</t>
+        </is>
+      </c>
+      <c r="L19" s="2" t="inlineStr">
+        <is>
+          <t>not confirmed</t>
+        </is>
+      </c>
+      <c r="M19" s="3" t="inlineStr">
+        <is>
+          <t>none found (checked @dr.pawpaw bio and @dr.pawpaw.hu, @dr.pawpaw.hungary, @dr.pawpaw.magyarorszag, @dr.pawpaw_hu, @dr.pawpaw_hungary, @dr.pawpawhu, @dr.pawpawhungary, @drpawpaw.hu, @drpawpaw.hungary, @drpawpaw.magyarorszag, @drpawpaw_hu, @drpawpaw_hungary, @drpawpawhu, @drpawpawhungary)</t>
+        </is>
+      </c>
+      <c r="N19" s="3" t="inlineStr"/>
       <c r="O19" s="3" t="inlineStr">
         <is>
-          <t>Your bronzing body and face balm with orange and cinnamon is exactly the kind of product that sells on TikTok: the glow is visible before and after in one short video.</t>
+          <t>Your Charm Balm Trio in banana, matcha and cherry is a colourful, giftable set that's easy to show in a short unboxing video.</t>
         </is>
       </c>
       <c r="P19" s="2" t="inlineStr">
@@ -1977,65 +1989,69 @@
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
         <is>
-          <t>Sylveco</t>
+          <t>Fable &amp; Mane</t>
         </is>
       </c>
       <c r="B20" s="2" t="inlineStr">
         <is>
-          <t>https://sylveco.pl/</t>
+          <t>https://fableandmane.com/</t>
         </is>
       </c>
       <c r="C20" s="2" t="inlineStr">
         <is>
-          <t>Poland</t>
+          <t>United Kingdom</t>
         </is>
       </c>
       <c r="D20" s="3" t="inlineStr">
         <is>
-          <t>https://sylveco.pl/regulamin/ — 'SYLVECO spółka z o.o. … z siedzibą w 36-004 Łąka k/Rzeszowa'</t>
+          <t>https://fableandmane.com/policies/terms-of-service — 'write to us at: 30-31 Plympton Street, London, NW8 8AB'</t>
         </is>
       </c>
       <c r="E20" s="2" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>A</t>
         </is>
       </c>
       <c r="F20" s="2" t="inlineStr">
         <is>
-          <t>Beauty / natural skincare</t>
+          <t>Beauty / haircare</t>
         </is>
       </c>
       <c r="G20" s="3" t="inlineStr">
         <is>
-          <t>SYLVECO birch cream with betulin (Krem brzozowy z betuliną) 50ml</t>
+          <t>HoliRoots Pre-Wash Scalp &amp; Hair Oil</t>
         </is>
       </c>
       <c r="H20" s="2" t="inlineStr">
         <is>
-          <t>53,99 zł</t>
+          <t>$38 / £34</t>
         </is>
       </c>
       <c r="I20" s="2" t="inlineStr">
         <is>
-          <t>export@sylveco.pl</t>
+          <t>support@fableandmane.com</t>
         </is>
       </c>
       <c r="J20" s="2" t="inlineStr"/>
       <c r="K20" s="3" t="inlineStr">
         <is>
-          <t>none on site; @sylveco.pl is not a TikTok Shop seller account</t>
-        </is>
-      </c>
-      <c r="L20" s="2" t="inlineStr"/>
-      <c r="M20" s="3" t="inlineStr"/>
-      <c r="N20" s="3" t="inlineStr">
-        <is>
-          <t>Ships to Hungary: shipping price list on sylveco.pl includes 'Węgry'</t>
-        </is>
-      </c>
+          <t>TikTok profile @fableandmane is a TikTok Shop seller account (ttSeller)</t>
+        </is>
+      </c>
+      <c r="L20" s="2" t="inlineStr">
+        <is>
+          <t>not confirmed</t>
+        </is>
+      </c>
+      <c r="M20" s="3" t="inlineStr">
+        <is>
+          <t>none found (checked @fableandmane bio and @fableandmane.hu, @fableandmane.hungary, @fableandmane.magyarorszag, @fableandmane_hu, @fableandmane_hungary, @fableandmanehu, @fableandmanehungary, @fablemane.hu, @fablemane.hungary, @fablemane.magyarorszag, @fablemane_hu, @fablemane_hungary, @fablemanehu, @fablemanehungary)</t>
+        </is>
+      </c>
+      <c r="N20" s="3" t="inlineStr"/>
       <c r="O20" s="3" t="inlineStr">
         <is>
-          <t>Your birch cream with betulin, one of your bestsellers, is a simple product to show in a short skincare video, with a natural-ingredient story creators can explain in seconds.</t>
+          <t>Your HoliRoots pre-wash scalp and hair oil is an easy product to demonstrate in a short wash-day routine video.</t>
         </is>
       </c>
       <c r="P20" s="2" t="inlineStr">
@@ -2045,6 +2061,1502 @@
       </c>
       <c r="Q20" s="3" t="inlineStr"/>
       <c r="R20" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-26</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="2" t="inlineStr">
+        <is>
+          <t>Glow Hub</t>
+        </is>
+      </c>
+      <c r="B21" s="2" t="inlineStr">
+        <is>
+          <t>https://glowhub.com/</t>
+        </is>
+      </c>
+      <c r="C21" s="2" t="inlineStr">
+        <is>
+          <t>United Kingdom</t>
+        </is>
+      </c>
+      <c r="D21" s="3" t="inlineStr">
+        <is>
+          <t>https://glowhub.com/pages/terms-conditions — 'registered in England and Wales … Knutsford, Cheshire, WA16 8ZR' (Amelia Knight Ltd)</t>
+        </is>
+      </c>
+      <c r="E21" s="2" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="F21" s="2" t="inlineStr">
+        <is>
+          <t>Beauty / skincare &amp; makeup</t>
+        </is>
+      </c>
+      <c r="G21" s="3" t="inlineStr">
+        <is>
+          <t>BABY BEAM dew filter glow base</t>
+        </is>
+      </c>
+      <c r="H21" s="2" t="inlineStr">
+        <is>
+          <t>£11.20</t>
+        </is>
+      </c>
+      <c r="I21" s="2" t="inlineStr">
+        <is>
+          <t>hello@glowhub.com</t>
+        </is>
+      </c>
+      <c r="J21" s="2" t="inlineStr"/>
+      <c r="K21" s="3" t="inlineStr">
+        <is>
+          <t>Site T&amp;Cs mention 'Glow Hub's TikTok shop'; TikTok profile @glowhubbeauty is a TikTok Shop seller account (ttSeller)</t>
+        </is>
+      </c>
+      <c r="L21" s="2" t="inlineStr">
+        <is>
+          <t>not confirmed</t>
+        </is>
+      </c>
+      <c r="M21" s="3" t="inlineStr">
+        <is>
+          <t>none found (checked @glowhubbeauty bio and @glowhub.hu, @glowhub.hungary, @glowhub.magyarorszag, @glowhub_hu, @glowhub_hungary, @glowhubbeauty.hu, @glowhubbeauty.hungary, @glowhubbeauty.magyarorszag, @glowhubbeauty_hu, @glowhubbeauty_hungary, @glowhubbeautyhu, @glowhubbeautyhungary, @glowhubhu, @glowhubhungary)</t>
+        </is>
+      </c>
+      <c r="N21" s="3" t="inlineStr"/>
+      <c r="O21" s="3" t="inlineStr">
+        <is>
+          <t>Your BABY BEAM dew filter glow base is exactly the kind of product that sells in a 15-second before-and-after video, because a dewy finish is easy to show on camera.</t>
+        </is>
+      </c>
+      <c r="P21" s="2" t="inlineStr">
+        <is>
+          <t>beauty and skincare creators</t>
+        </is>
+      </c>
+      <c r="Q21" s="3" t="inlineStr"/>
+      <c r="R21" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-26</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="2" t="inlineStr">
+        <is>
+          <t>Hair Syrup</t>
+        </is>
+      </c>
+      <c r="B22" s="2" t="inlineStr">
+        <is>
+          <t>https://hairsyrup.co.uk/</t>
+        </is>
+      </c>
+      <c r="C22" s="2" t="inlineStr">
+        <is>
+          <t>United Kingdom</t>
+        </is>
+      </c>
+      <c r="D22" s="3" t="inlineStr">
+        <is>
+          <t>https://hairsyrup.co.uk/policies/terms-of-service — 'laws of United Kingdom'; privacy policy: 'Hair Syrup Ltd, … Fishguard SA65 9NG'</t>
+        </is>
+      </c>
+      <c r="E22" s="2" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="F22" s="2" t="inlineStr">
+        <is>
+          <t>Beauty / haircare</t>
+        </is>
+      </c>
+      <c r="G22" s="3" t="inlineStr">
+        <is>
+          <t>Watermelon Oil pre-wash hair oil</t>
+        </is>
+      </c>
+      <c r="H22" s="2" t="inlineStr">
+        <is>
+          <t>£16.95</t>
+        </is>
+      </c>
+      <c r="I22" s="2" t="inlineStr">
+        <is>
+          <t>hello@hairsyrup.co.uk</t>
+        </is>
+      </c>
+      <c r="J22" s="2" t="inlineStr"/>
+      <c r="K22" s="3" t="inlineStr">
+        <is>
+          <t>TikTok profile @hairsyrup is a TikTok Shop seller account (ttSeller)</t>
+        </is>
+      </c>
+      <c r="L22" s="2" t="inlineStr">
+        <is>
+          <t>not confirmed</t>
+        </is>
+      </c>
+      <c r="M22" s="3" t="inlineStr">
+        <is>
+          <t>none found (checked @hairsyrup bio and @hairsyrup.hu, @hairsyrup.hungary, @hairsyrup.magyarorszag, @hairsyrup_hu, @hairsyrup_hungary, @hairsyruphu, @hairsyruphungary)</t>
+        </is>
+      </c>
+      <c r="N22" s="3" t="inlineStr"/>
+      <c r="O22" s="3" t="inlineStr">
+        <is>
+          <t>Your Watermelon Oil, first in your best sellers, is a pre-wash hair oil that's easy to show in a short wash-day video, from applying it to the finished hair.</t>
+        </is>
+      </c>
+      <c r="P22" s="2" t="inlineStr">
+        <is>
+          <t>beauty and skincare creators</t>
+        </is>
+      </c>
+      <c r="Q22" s="3" t="inlineStr"/>
+      <c r="R22" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-26</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="2" t="inlineStr">
+        <is>
+          <t>Hairburst</t>
+        </is>
+      </c>
+      <c r="B23" s="2" t="inlineStr">
+        <is>
+          <t>https://www.hairburst.com/</t>
+        </is>
+      </c>
+      <c r="C23" s="2" t="inlineStr">
+        <is>
+          <t>United Kingdom</t>
+        </is>
+      </c>
+      <c r="D23" s="3" t="inlineStr">
+        <is>
+          <t>https://www.hairburst.com/pages/terms-of-service — 'Registered in England with company number 08898301'</t>
+        </is>
+      </c>
+      <c r="E23" s="2" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="F23" s="2" t="inlineStr">
+        <is>
+          <t>Beauty / haircare</t>
+        </is>
+      </c>
+      <c r="G23" s="3" t="inlineStr">
+        <is>
+          <t>Chewable Hair Vitamins (hair gummies)</t>
+        </is>
+      </c>
+      <c r="H23" s="2" t="inlineStr">
+        <is>
+          <t>£22.99 (1 month)</t>
+        </is>
+      </c>
+      <c r="I23" s="2" t="inlineStr">
+        <is>
+          <t>support@hairburst.com</t>
+        </is>
+      </c>
+      <c r="J23" s="2" t="inlineStr"/>
+      <c r="K23" s="3" t="inlineStr">
+        <is>
+          <t>TikTok profile @hairburst is a TikTok Shop seller account (ttSeller)</t>
+        </is>
+      </c>
+      <c r="L23" s="2" t="inlineStr">
+        <is>
+          <t>not confirmed</t>
+        </is>
+      </c>
+      <c r="M23" s="3" t="inlineStr">
+        <is>
+          <t>none found (checked @hairburst bio and @hairburst.hu, @hairburst.hungary, @hairburst.magyarorszag, @hairburst_hu, @hairburst_hungary, @hairbursthu, @hairbursthungary)</t>
+        </is>
+      </c>
+      <c r="N23" s="3" t="inlineStr">
+        <is>
+          <t>Hungarian site version hairburst.com/hu-hu</t>
+        </is>
+      </c>
+      <c r="O23" s="3" t="inlineStr">
+        <is>
+          <t>Your chewable hair vitamins are an easy daily habit to film, and a hair routine gives creators a natural reason to post updates over several weeks.</t>
+        </is>
+      </c>
+      <c r="P23" s="2" t="inlineStr">
+        <is>
+          <t>beauty and skincare creators</t>
+        </is>
+      </c>
+      <c r="Q23" s="3" t="inlineStr"/>
+      <c r="R23" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-26</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="2" t="inlineStr">
+        <is>
+          <t>Nails.INC</t>
+        </is>
+      </c>
+      <c r="B24" s="2" t="inlineStr">
+        <is>
+          <t>https://nailsinc.com/</t>
+        </is>
+      </c>
+      <c r="C24" s="2" t="inlineStr">
+        <is>
+          <t>United Kingdom</t>
+        </is>
+      </c>
+      <c r="D24" s="3" t="inlineStr">
+        <is>
+          <t>https://nailsinc.com/policies/privacy-policy — '19-23 Grosvenor Hill, London W1K 3QD, United Kingdom'</t>
+        </is>
+      </c>
+      <c r="E24" s="2" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="F24" s="2" t="inlineStr">
+        <is>
+          <t>Beauty / nails</t>
+        </is>
+      </c>
+      <c r="G24" s="3" t="inlineStr">
+        <is>
+          <t>45 Second Speedy Gloss nail polish duo</t>
+        </is>
+      </c>
+      <c r="H24" s="2" t="inlineStr">
+        <is>
+          <t>£15</t>
+        </is>
+      </c>
+      <c r="I24" s="2" t="inlineStr">
+        <is>
+          <t>hello@nailsinc.com</t>
+        </is>
+      </c>
+      <c r="J24" s="2" t="inlineStr"/>
+      <c r="K24" s="3" t="inlineStr">
+        <is>
+          <t>TikTok profile @nailsinclondon is a TikTok Shop seller account (ttSeller)</t>
+        </is>
+      </c>
+      <c r="L24" s="2" t="inlineStr">
+        <is>
+          <t>not confirmed</t>
+        </is>
+      </c>
+      <c r="M24" s="3" t="inlineStr">
+        <is>
+          <t>none found (checked @nailsinclondon bio and @nailsinc.hu, @nailsinc.hungary, @nailsinc.magyarorszag, @nailsinc_hu, @nailsinc_hungary, @nailsinchu, @nailsinchungary, @nailsinclondon.hu, @nailsinclondon.hungary, @nailsinclondon.magyarorszag, @nailsinclondon_hu, @nailsinclondon_hungary, @nailsinclondonhu, @nailsinclondonhungary)</t>
+        </is>
+      </c>
+      <c r="N24" s="3" t="inlineStr"/>
+      <c r="O24" s="3" t="inlineStr">
+        <is>
+          <t>Your 45 Second Speedy Gloss nail polish duos are made for short videos: the quick-dry promise in the name is something creators can show on camera in real time.</t>
+        </is>
+      </c>
+      <c r="P24" s="2" t="inlineStr">
+        <is>
+          <t>beauty and skincare creators</t>
+        </is>
+      </c>
+      <c r="Q24" s="3" t="inlineStr"/>
+      <c r="R24" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-26</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="2" t="inlineStr">
+        <is>
+          <t>Nala's Baby</t>
+        </is>
+      </c>
+      <c r="B25" s="2" t="inlineStr">
+        <is>
+          <t>https://nalasbaby.com/</t>
+        </is>
+      </c>
+      <c r="C25" s="2" t="inlineStr">
+        <is>
+          <t>United Kingdom</t>
+        </is>
+      </c>
+      <c r="D25" s="3" t="inlineStr">
+        <is>
+          <t>https://nalasbaby.com/pages/terms-conditions — 'governed by … the laws of England and Wales'</t>
+        </is>
+      </c>
+      <c r="E25" s="2" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="F25" s="2" t="inlineStr">
+        <is>
+          <t>Baby / kids care</t>
+        </is>
+      </c>
+      <c r="G25" s="3" t="inlineStr">
+        <is>
+          <t>Nala's Baby Bath-time Gift Set</t>
+        </is>
+      </c>
+      <c r="H25" s="2" t="inlineStr">
+        <is>
+          <t>£25.99</t>
+        </is>
+      </c>
+      <c r="I25" s="2" t="inlineStr">
+        <is>
+          <t>info@nalasbaby.com</t>
+        </is>
+      </c>
+      <c r="J25" s="2" t="inlineStr"/>
+      <c r="K25" s="3" t="inlineStr">
+        <is>
+          <t>TikTok profile @nalasbaby is a TikTok Shop seller account (ttSeller) named "Nala's Baby UK"</t>
+        </is>
+      </c>
+      <c r="L25" s="2" t="inlineStr">
+        <is>
+          <t>not confirmed</t>
+        </is>
+      </c>
+      <c r="M25" s="3" t="inlineStr">
+        <is>
+          <t>none found (checked @nalasbaby bio and @nalasbaby.hu, @nalasbaby.hungary, @nalasbaby.magyarorszag, @nalasbaby_hu, @nalasbaby_hungary, @nalasbabyhu, @nalasbabyhungary)</t>
+        </is>
+      </c>
+      <c r="N25" s="3" t="inlineStr"/>
+      <c r="O25" s="3" t="inlineStr">
+        <is>
+          <t>Your Bath-time Gift Set is a ready-made, giftable bundle, and bath time is one of the easiest family moments to show in a short video.</t>
+        </is>
+      </c>
+      <c r="P25" s="2" t="inlineStr">
+        <is>
+          <t>home and lifestyle creators</t>
+        </is>
+      </c>
+      <c r="Q25" s="3" t="inlineStr"/>
+      <c r="R25" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-26</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="2" t="inlineStr">
+        <is>
+          <t>Nip+Fab</t>
+        </is>
+      </c>
+      <c r="B26" s="2" t="inlineStr">
+        <is>
+          <t>https://www.nipandfab.com/</t>
+        </is>
+      </c>
+      <c r="C26" s="2" t="inlineStr">
+        <is>
+          <t>United Kingdom</t>
+        </is>
+      </c>
+      <c r="D26" s="3" t="inlineStr">
+        <is>
+          <t>https://www.nipandfab.com/pages/terms-conditions — 'Nip and Fab Limited … Registered office: … 21 Evesham Street, London W11 4AJ'</t>
+        </is>
+      </c>
+      <c r="E26" s="2" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="F26" s="2" t="inlineStr">
+        <is>
+          <t>Beauty / skincare</t>
+        </is>
+      </c>
+      <c r="G26" s="3" t="inlineStr">
+        <is>
+          <t>Award-Winning Duo - Peptides &amp; Ceramides</t>
+        </is>
+      </c>
+      <c r="H26" s="2" t="inlineStr">
+        <is>
+          <t>£39.95</t>
+        </is>
+      </c>
+      <c r="I26" s="2" t="inlineStr">
+        <is>
+          <t>enquiries@nipandfab.com</t>
+        </is>
+      </c>
+      <c r="J26" s="2" t="inlineStr"/>
+      <c r="K26" s="3" t="inlineStr">
+        <is>
+          <t>TikTok profile @nipandfab is a TikTok Shop seller account (ttSeller)</t>
+        </is>
+      </c>
+      <c r="L26" s="2" t="inlineStr">
+        <is>
+          <t>not confirmed</t>
+        </is>
+      </c>
+      <c r="M26" s="3" t="inlineStr">
+        <is>
+          <t>none found (checked @nipandfab bio and @nipandfab.hu, @nipandfab.hungary, @nipandfab.magyarorszag, @nipandfab_hu, @nipandfab_hungary, @nipandfabhu, @nipandfabhungary, @nipfab.hu, @nipfab.hungary, @nipfab.magyarorszag, @nipfab_hu, @nipfab_hungary, @nipfabhu, @nipfabhungary)</t>
+        </is>
+      </c>
+      <c r="N26" s="3" t="inlineStr"/>
+      <c r="O26" s="3" t="inlineStr">
+        <is>
+          <t>Your Award-Winning Duo of peptides and ceramides is easy to show in a short routine video, and a two-step set gives creators a simple routine to film.</t>
+        </is>
+      </c>
+      <c r="P26" s="2" t="inlineStr">
+        <is>
+          <t>beauty and skincare creators</t>
+        </is>
+      </c>
+      <c r="Q26" s="3" t="inlineStr"/>
+      <c r="R26" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-26</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="2" t="inlineStr">
+        <is>
+          <t>Novomins</t>
+        </is>
+      </c>
+      <c r="B27" s="2" t="inlineStr">
+        <is>
+          <t>https://novomins.com/</t>
+        </is>
+      </c>
+      <c r="C27" s="2" t="inlineStr">
+        <is>
+          <t>United Kingdom</t>
+        </is>
+      </c>
+      <c r="D27" s="3" t="inlineStr">
+        <is>
+          <t>https://novomins.com/policies/terms-of-service — 'operated by Innocent Health Ltd … laws of England and Wales'</t>
+        </is>
+      </c>
+      <c r="E27" s="2" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="F27" s="2" t="inlineStr">
+        <is>
+          <t>Supplements / beauty</t>
+        </is>
+      </c>
+      <c r="G27" s="3" t="inlineStr">
+        <is>
+          <t>Collagen Gummies (Best Seller)</t>
+        </is>
+      </c>
+      <c r="H27" s="2" t="inlineStr">
+        <is>
+          <t>£19.99</t>
+        </is>
+      </c>
+      <c r="I27" s="2" t="inlineStr">
+        <is>
+          <t>hello@novomins.com</t>
+        </is>
+      </c>
+      <c r="J27" s="2" t="inlineStr"/>
+      <c r="K27" s="3" t="inlineStr">
+        <is>
+          <t>TikTok profile @novominsnutrition is a TikTok Shop seller account (ttSeller)</t>
+        </is>
+      </c>
+      <c r="L27" s="2" t="inlineStr">
+        <is>
+          <t>not confirmed</t>
+        </is>
+      </c>
+      <c r="M27" s="3" t="inlineStr">
+        <is>
+          <t>none found (checked @novominsnutrition bio and @novomins.hu, @novomins.hungary, @novomins.magyarorszag, @novomins_hu, @novomins_hungary, @novominshu, @novominshungary, @novominsnutrition.hu, @novominsnutrition.hungary, @novominsnutrition.magyarorszag, @novominsnutrition_hu, @novominsnutrition_hungary, @novominsnutritionhu, @novominsnutritionhungary)</t>
+        </is>
+      </c>
+      <c r="N27" s="3" t="inlineStr"/>
+      <c r="O27" s="3" t="inlineStr">
+        <is>
+          <t>Your Collagen Gummies, marked Best Seller on your site, are an easy daily habit to film, and gummies are far more fun on camera than a capsule.</t>
+        </is>
+      </c>
+      <c r="P27" s="2" t="inlineStr">
+        <is>
+          <t>beauty and skincare creators</t>
+        </is>
+      </c>
+      <c r="Q27" s="3" t="inlineStr"/>
+      <c r="R27" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-26</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="2" t="inlineStr">
+        <is>
+          <t>Orelia</t>
+        </is>
+      </c>
+      <c r="B28" s="2" t="inlineStr">
+        <is>
+          <t>https://orelia.com/</t>
+        </is>
+      </c>
+      <c r="C28" s="2" t="inlineStr">
+        <is>
+          <t>United Kingdom</t>
+        </is>
+      </c>
+      <c r="D28" s="3" t="inlineStr">
+        <is>
+          <t>https://orelia.com/pages/terms-and-condition — 'Orelia Ltd, 21 Hambridge Trading Estate, … Worthing, West Sussex, BN14 8NA'</t>
+        </is>
+      </c>
+      <c r="E28" s="2" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="F28" s="2" t="inlineStr">
+        <is>
+          <t>Jewellery</t>
+        </is>
+      </c>
+      <c r="G28" s="3" t="inlineStr">
+        <is>
+          <t>Pavé &amp; Pearl Drop Ear Stacking Set</t>
+        </is>
+      </c>
+      <c r="H28" s="2" t="inlineStr">
+        <is>
+          <t>£42</t>
+        </is>
+      </c>
+      <c r="I28" s="2" t="inlineStr">
+        <is>
+          <t>info@orelia.co.uk</t>
+        </is>
+      </c>
+      <c r="J28" s="2" t="inlineStr"/>
+      <c r="K28" s="3" t="inlineStr">
+        <is>
+          <t>TikTok profile @oreliajewellery is a TikTok Shop seller account (ttSeller)</t>
+        </is>
+      </c>
+      <c r="L28" s="2" t="inlineStr">
+        <is>
+          <t>not confirmed</t>
+        </is>
+      </c>
+      <c r="M28" s="3" t="inlineStr">
+        <is>
+          <t>none found (checked @oreliajewellery bio and @orelia.hu, @orelia.hungary, @orelia.magyarorszag, @orelia_hu, @orelia_hungary, @oreliahu, @oreliahungary, @oreliajewellery.hu, @oreliajewellery.hungary, @oreliajewellery.magyarorszag, @oreliajewellery_hu, @oreliajewellery_hungary, @oreliajewelleryhu, @oreliajewelleryhungary)</t>
+        </is>
+      </c>
+      <c r="N28" s="3" t="inlineStr"/>
+      <c r="O28" s="3" t="inlineStr">
+        <is>
+          <t>Your Pavé &amp; Pearl Drop Ear Stacking Set is made for try-on videos where creators build the stack piece by piece, and it's an easy gift to show.</t>
+        </is>
+      </c>
+      <c r="P28" s="2" t="inlineStr">
+        <is>
+          <t>fashion and accessories creators</t>
+        </is>
+      </c>
+      <c r="Q28" s="3" t="inlineStr"/>
+      <c r="R28" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-26</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="2" t="inlineStr">
+        <is>
+          <t>Pet Munchies</t>
+        </is>
+      </c>
+      <c r="B29" s="2" t="inlineStr">
+        <is>
+          <t>https://pet-munchies.com/</t>
+        </is>
+      </c>
+      <c r="C29" s="2" t="inlineStr">
+        <is>
+          <t>United Kingdom</t>
+        </is>
+      </c>
+      <c r="D29" s="3" t="inlineStr">
+        <is>
+          <t>https://pet-munchies.com/policies/terms-of-service — 'Pet Munchies Limited … registered in England and Wales'</t>
+        </is>
+      </c>
+      <c r="E29" s="2" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="F29" s="2" t="inlineStr">
+        <is>
+          <t>Pets</t>
+        </is>
+      </c>
+      <c r="G29" s="3" t="inlineStr">
+        <is>
+          <t>Training Treats Bundle - Venison, Salmon, Sushi</t>
+        </is>
+      </c>
+      <c r="H29" s="2" t="inlineStr">
+        <is>
+          <t>£29.99</t>
+        </is>
+      </c>
+      <c r="I29" s="2" t="inlineStr">
+        <is>
+          <t>hello@pet-munchies.com</t>
+        </is>
+      </c>
+      <c r="J29" s="2" t="inlineStr"/>
+      <c r="K29" s="3" t="inlineStr">
+        <is>
+          <t>TikTok profile @petmunchies is a TikTok Shop seller account (ttSeller)</t>
+        </is>
+      </c>
+      <c r="L29" s="2" t="inlineStr">
+        <is>
+          <t>not confirmed</t>
+        </is>
+      </c>
+      <c r="M29" s="3" t="inlineStr">
+        <is>
+          <t>none found (checked @petmunchies bio and @petmunchies.hu, @petmunchies.hungary, @petmunchies.magyarorszag, @petmunchies_hu, @petmunchies_hungary, @petmunchieshu, @petmunchieshungary)</t>
+        </is>
+      </c>
+      <c r="N29" s="3" t="inlineStr"/>
+      <c r="O29" s="3" t="inlineStr">
+        <is>
+          <t>Your Training Treats Bundle is made for short dog-training videos, one of the easiest kinds of pet content for creators to film.</t>
+        </is>
+      </c>
+      <c r="P29" s="2" t="inlineStr">
+        <is>
+          <t>pet and lifestyle creators</t>
+        </is>
+      </c>
+      <c r="Q29" s="3" t="inlineStr"/>
+      <c r="R29" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-26</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="2" t="inlineStr">
+        <is>
+          <t>Pets Purest</t>
+        </is>
+      </c>
+      <c r="B30" s="2" t="inlineStr">
+        <is>
+          <t>https://www.petspurest.com/</t>
+        </is>
+      </c>
+      <c r="C30" s="2" t="inlineStr">
+        <is>
+          <t>United Kingdom</t>
+        </is>
+      </c>
+      <c r="D30" s="3" t="inlineStr">
+        <is>
+          <t>https://www.petspurest.com/policies/terms-of-service — 'OE Enterprises Limited, … Lymm, Cheshire, WA13 0SU, United Kingdom'</t>
+        </is>
+      </c>
+      <c r="E30" s="2" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="F30" s="2" t="inlineStr">
+        <is>
+          <t>Pets</t>
+        </is>
+      </c>
+      <c r="G30" s="3" t="inlineStr">
+        <is>
+          <t>Natural Scottish Salmon Oil for Dogs &amp; Cats (1000ml)</t>
+        </is>
+      </c>
+      <c r="H30" s="2" t="inlineStr">
+        <is>
+          <t>£19.99</t>
+        </is>
+      </c>
+      <c r="I30" s="2" t="inlineStr">
+        <is>
+          <t>info@petspurest.com</t>
+        </is>
+      </c>
+      <c r="J30" s="2" t="inlineStr"/>
+      <c r="K30" s="3" t="inlineStr">
+        <is>
+          <t>TikTok profile @petspurest is a TikTok Shop seller account (ttSeller)</t>
+        </is>
+      </c>
+      <c r="L30" s="2" t="inlineStr">
+        <is>
+          <t>not confirmed</t>
+        </is>
+      </c>
+      <c r="M30" s="3" t="inlineStr">
+        <is>
+          <t>none found (checked @petspurest bio and @petspurest.hu, @petspurest.hungary, @petspurest.magyarorszag, @petspurest_hu, @petspurest_hungary, @petspuresthu, @petspuresthungary)</t>
+        </is>
+      </c>
+      <c r="N30" s="3" t="inlineStr"/>
+      <c r="O30" s="3" t="inlineStr">
+        <is>
+          <t>Your Natural Scottish Salmon Oil for dogs and cats is easy to show in a short video: one pump over the bowl at feeding time, a moment pet owners film anyway.</t>
+        </is>
+      </c>
+      <c r="P30" s="2" t="inlineStr">
+        <is>
+          <t>pet and lifestyle creators</t>
+        </is>
+      </c>
+      <c r="Q30" s="3" t="inlineStr"/>
+      <c r="R30" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-26</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="2" t="inlineStr">
+        <is>
+          <t>Skin &amp; Tan</t>
+        </is>
+      </c>
+      <c r="B31" s="2" t="inlineStr">
+        <is>
+          <t>https://www.skinandtan.co.uk/</t>
+        </is>
+      </c>
+      <c r="C31" s="2" t="inlineStr">
+        <is>
+          <t>United Kingdom</t>
+        </is>
+      </c>
+      <c r="D31" s="3" t="inlineStr">
+        <is>
+          <t>https://www.skinandtan.co.uk/pages/terms-and-conditions — 'The Brand Architekts Limited trading as Skin &amp; Tan … Iver, Buckinghamshire, SL0 9HW'</t>
+        </is>
+      </c>
+      <c r="E31" s="2" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="F31" s="2" t="inlineStr">
+        <is>
+          <t>Beauty / self-tan</t>
+        </is>
+      </c>
+      <c r="G31" s="3" t="inlineStr">
+        <is>
+          <t>Self-Tanning Mousse 150ml</t>
+        </is>
+      </c>
+      <c r="H31" s="2" t="inlineStr">
+        <is>
+          <t>£21.99</t>
+        </is>
+      </c>
+      <c r="I31" s="2" t="inlineStr">
+        <is>
+          <t>info@skinandtan.com</t>
+        </is>
+      </c>
+      <c r="J31" s="2" t="inlineStr"/>
+      <c r="K31" s="3" t="inlineStr">
+        <is>
+          <t>TikTok profile @skinandtan is a TikTok Shop seller account (ttSeller)</t>
+        </is>
+      </c>
+      <c r="L31" s="2" t="inlineStr">
+        <is>
+          <t>not confirmed</t>
+        </is>
+      </c>
+      <c r="M31" s="3" t="inlineStr">
+        <is>
+          <t>none found (checked @skinandtan bio and @skinandtan.hu, @skinandtan.hungary, @skinandtan.magyarorszag, @skinandtan_hu, @skinandtan_hungary, @skinandtanhu, @skinandtanhungary, @skintan.hu, @skintan.hungary, @skintan.magyarorszag, @skintan_hu, @skintan_hungary, @skintanhu, @skintanhungary)</t>
+        </is>
+      </c>
+      <c r="N31" s="3" t="inlineStr"/>
+      <c r="O31" s="3" t="inlineStr">
+        <is>
+          <t>Your Self-Tanning Mousse is exactly the kind of product that sells on TikTok: the difference between before and after is visible in one short video.</t>
+        </is>
+      </c>
+      <c r="P31" s="2" t="inlineStr">
+        <is>
+          <t>beauty and skincare creators</t>
+        </is>
+      </c>
+      <c r="Q31" s="3" t="inlineStr"/>
+      <c r="R31" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-26</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="2" t="inlineStr">
+        <is>
+          <t>Tangle Angel</t>
+        </is>
+      </c>
+      <c r="B32" s="2" t="inlineStr">
+        <is>
+          <t>https://tangleangel.com/</t>
+        </is>
+      </c>
+      <c r="C32" s="2" t="inlineStr">
+        <is>
+          <t>United Kingdom</t>
+        </is>
+      </c>
+      <c r="D32" s="3" t="inlineStr">
+        <is>
+          <t>https://tangleangel.com/policies/terms-of-service — 'Tangle Angel Limited, Registered in England … 1 Duchess Street, London W1W 6AN'</t>
+        </is>
+      </c>
+      <c r="E32" s="2" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="F32" s="2" t="inlineStr">
+        <is>
+          <t>Beauty / hair tools</t>
+        </is>
+      </c>
+      <c r="G32" s="3" t="inlineStr">
+        <is>
+          <t>ANGEL 2.0 detangling brush</t>
+        </is>
+      </c>
+      <c r="H32" s="2" t="inlineStr">
+        <is>
+          <t>£15</t>
+        </is>
+      </c>
+      <c r="I32" s="2" t="inlineStr">
+        <is>
+          <t>info@tangleangel.com</t>
+        </is>
+      </c>
+      <c r="J32" s="2" t="inlineStr"/>
+      <c r="K32" s="3" t="inlineStr">
+        <is>
+          <t>TikTok profile @tangleangel is a TikTok Shop seller account (ttSeller)</t>
+        </is>
+      </c>
+      <c r="L32" s="2" t="inlineStr">
+        <is>
+          <t>not confirmed</t>
+        </is>
+      </c>
+      <c r="M32" s="3" t="inlineStr">
+        <is>
+          <t>none found (checked @tangleangel bio and @tangleangel.hu, @tangleangel.hungary, @tangleangel.magyarorszag, @tangleangel_hu, @tangleangel_hungary, @tangleangelhu, @tangleangelhungary)</t>
+        </is>
+      </c>
+      <c r="N32" s="3" t="inlineStr"/>
+      <c r="O32" s="3" t="inlineStr">
+        <is>
+          <t>Your ANGEL 2.0 detangling brush is exactly the kind of product that sells in a 15-second demo video: one pass through knotted hair shows the result.</t>
+        </is>
+      </c>
+      <c r="P32" s="2" t="inlineStr">
+        <is>
+          <t>beauty and skincare creators</t>
+        </is>
+      </c>
+      <c r="Q32" s="3" t="inlineStr"/>
+      <c r="R32" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-26</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="2" t="inlineStr">
+        <is>
+          <t>UpCircle</t>
+        </is>
+      </c>
+      <c r="B33" s="2" t="inlineStr">
+        <is>
+          <t>https://upcirclebeauty.com/</t>
+        </is>
+      </c>
+      <c r="C33" s="2" t="inlineStr">
+        <is>
+          <t>United Kingdom</t>
+        </is>
+      </c>
+      <c r="D33" s="3" t="inlineStr">
+        <is>
+          <t>https://upcirclebeauty.com/policies/terms-of-service — 'operated by Optiat Ltd … laws of Unit 8, Uplands Business Park, London E17 5QJ'</t>
+        </is>
+      </c>
+      <c r="E33" s="2" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="F33" s="2" t="inlineStr">
+        <is>
+          <t>Beauty / skincare</t>
+        </is>
+      </c>
+      <c r="G33" s="3" t="inlineStr">
+        <is>
+          <t>Powder to Foam Face Wash with Willow Bark + Papaya Enzymes</t>
+        </is>
+      </c>
+      <c r="H33" s="2" t="inlineStr">
+        <is>
+          <t>£21.99</t>
+        </is>
+      </c>
+      <c r="I33" s="2" t="inlineStr">
+        <is>
+          <t>hello@upcirclebeauty.com</t>
+        </is>
+      </c>
+      <c r="J33" s="2" t="inlineStr"/>
+      <c r="K33" s="3" t="inlineStr">
+        <is>
+          <t>TikTok profile @upcirclebeauty is a TikTok Shop seller account (ttSeller)</t>
+        </is>
+      </c>
+      <c r="L33" s="2" t="inlineStr">
+        <is>
+          <t>not confirmed</t>
+        </is>
+      </c>
+      <c r="M33" s="3" t="inlineStr">
+        <is>
+          <t>none found (checked @upcirclebeauty bio and @upcircle.hu, @upcircle_hu, @upcirclehu, @upcircle.hungary …)</t>
+        </is>
+      </c>
+      <c r="N33" s="3" t="inlineStr"/>
+      <c r="O33" s="3" t="inlineStr">
+        <is>
+          <t>Your Powder to Foam Face Wash is made for a short video: the moment the powder turns into foam in your hands is the kind of demo that sells on TikTok.</t>
+        </is>
+      </c>
+      <c r="P33" s="2" t="inlineStr">
+        <is>
+          <t>beauty and skincare creators</t>
+        </is>
+      </c>
+      <c r="Q33" s="3" t="inlineStr"/>
+      <c r="R33" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-26</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="2" t="inlineStr">
+        <is>
+          <t>Vieve</t>
+        </is>
+      </c>
+      <c r="B34" s="2" t="inlineStr">
+        <is>
+          <t>https://www.vievebeauty.com/</t>
+        </is>
+      </c>
+      <c r="C34" s="2" t="inlineStr">
+        <is>
+          <t>United Kingdom</t>
+        </is>
+      </c>
+      <c r="D34" s="3" t="inlineStr">
+        <is>
+          <t>https://www.vievebeauty.com/pages/terms-and-conditions — 'incorporated in Scotland (17c Townhead Street, Strathaven … ML10 6AB)'</t>
+        </is>
+      </c>
+      <c r="E34" s="2" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="F34" s="2" t="inlineStr">
+        <is>
+          <t>Beauty / makeup</t>
+        </is>
+      </c>
+      <c r="G34" s="3" t="inlineStr">
+        <is>
+          <t>Skin Nova Complexion Balm</t>
+        </is>
+      </c>
+      <c r="H34" s="2" t="inlineStr">
+        <is>
+          <t>£36</t>
+        </is>
+      </c>
+      <c r="I34" s="2" t="inlineStr">
+        <is>
+          <t>support@vieve.co.uk</t>
+        </is>
+      </c>
+      <c r="J34" s="2" t="inlineStr"/>
+      <c r="K34" s="3" t="inlineStr">
+        <is>
+          <t>TikTok profile @vievemuse is a TikTok Shop seller account (ttSeller)</t>
+        </is>
+      </c>
+      <c r="L34" s="2" t="inlineStr">
+        <is>
+          <t>not confirmed</t>
+        </is>
+      </c>
+      <c r="M34" s="3" t="inlineStr">
+        <is>
+          <t>none found (checked @vievemuse bio and @vieve.hu, @vieve.hungary, @vieve.magyarorszag, @vieve_hu, @vieve_hungary, @vievehu, @vievehungary, @vievemuse.hu, @vievemuse.hungary, @vievemuse.magyarorszag, @vievemuse_hu, @vievemuse_hungary, @vievemusehu, @vievemusehungary)</t>
+        </is>
+      </c>
+      <c r="N34" s="3" t="inlineStr"/>
+      <c r="O34" s="3" t="inlineStr">
+        <is>
+          <t>Your Skin Nova Complexion Balm is easy to demonstrate in a short video: half the face with it, half without, in one short clip.</t>
+        </is>
+      </c>
+      <c r="P34" s="2" t="inlineStr">
+        <is>
+          <t>beauty and skincare creators</t>
+        </is>
+      </c>
+      <c r="Q34" s="3" t="inlineStr"/>
+      <c r="R34" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-26</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="2" t="inlineStr">
+        <is>
+          <t>Clochee</t>
+        </is>
+      </c>
+      <c r="B35" s="2" t="inlineStr">
+        <is>
+          <t>https://www.clochee.com/</t>
+        </is>
+      </c>
+      <c r="C35" s="2" t="inlineStr">
+        <is>
+          <t>Poland</t>
+        </is>
+      </c>
+      <c r="D35" s="3" t="inlineStr">
+        <is>
+          <t>https://www.clochee.com/en/terms — 'Clochee Sp. z o o … Szczecin (POLAND)'</t>
+        </is>
+      </c>
+      <c r="E35" s="2" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="F35" s="2" t="inlineStr">
+        <is>
+          <t>Natural cosmetics</t>
+        </is>
+      </c>
+      <c r="G35" s="3" t="inlineStr"/>
+      <c r="H35" s="2" t="inlineStr"/>
+      <c r="I35" s="2" t="inlineStr">
+        <is>
+          <t>sklep@clochee.com</t>
+        </is>
+      </c>
+      <c r="J35" s="2" t="inlineStr"/>
+      <c r="K35" s="3" t="inlineStr">
+        <is>
+          <t>none on site; TikTok profile not a seller account</t>
+        </is>
+      </c>
+      <c r="L35" s="2" t="inlineStr"/>
+      <c r="M35" s="3" t="inlineStr"/>
+      <c r="N35" s="3" t="inlineStr">
+        <is>
+          <t>Hungary (Węgry) in shipping country selector</t>
+        </is>
+      </c>
+      <c r="O35" s="3" t="inlineStr"/>
+      <c r="P35" s="2" t="inlineStr">
+        <is>
+          <t>beauty and skincare creators</t>
+        </is>
+      </c>
+      <c r="Q35" s="3" t="inlineStr">
+        <is>
+          <t>no specific opener found on site; no featured product; no specific featured product found on site</t>
+        </is>
+      </c>
+      <c r="R35" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-26</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="2" t="inlineStr">
+        <is>
+          <t>Makear</t>
+        </is>
+      </c>
+      <c r="B36" s="2" t="inlineStr">
+        <is>
+          <t>https://makear.pl/</t>
+        </is>
+      </c>
+      <c r="C36" s="2" t="inlineStr">
+        <is>
+          <t>Poland</t>
+        </is>
+      </c>
+      <c r="D36" s="3" t="inlineStr">
+        <is>
+          <t>https://makear.pl/pl/terms.html — 'Adres siedziby Sprzedającego: Krzysztofa Kolumba 9B, 51-503 Wrocław'</t>
+        </is>
+      </c>
+      <c r="E36" s="2" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="F36" s="2" t="inlineStr">
+        <is>
+          <t>Beauty / nails</t>
+        </is>
+      </c>
+      <c r="G36" s="3" t="inlineStr">
+        <is>
+          <t>NEONS UV gel polish (glow in the dark)</t>
+        </is>
+      </c>
+      <c r="H36" s="2" t="inlineStr">
+        <is>
+          <t>~10 € (8 ml)</t>
+        </is>
+      </c>
+      <c r="I36" s="2" t="inlineStr">
+        <is>
+          <t>info@makear.pl</t>
+        </is>
+      </c>
+      <c r="J36" s="2" t="inlineStr"/>
+      <c r="K36" s="3" t="inlineStr">
+        <is>
+          <t>none on site; @makear is not a TikTok Shop seller account</t>
+        </is>
+      </c>
+      <c r="L36" s="2" t="inlineStr"/>
+      <c r="M36" s="3" t="inlineStr"/>
+      <c r="N36" s="3" t="inlineStr">
+        <is>
+          <t>Ships to Hungary: 'Country of collecting the order' list on makear.pl includes Hungary</t>
+        </is>
+      </c>
+      <c r="O36" s="3" t="inlineStr">
+        <is>
+          <t>Your NEONS UV gel polishes glow in the dark, which is exactly the kind of effect that sells in a 15-second video: lights off, and the result is on screen.</t>
+        </is>
+      </c>
+      <c r="P36" s="2" t="inlineStr">
+        <is>
+          <t>beauty and skincare creators</t>
+        </is>
+      </c>
+      <c r="Q36" s="3" t="inlineStr"/>
+      <c r="R36" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-26</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="2" t="inlineStr">
+        <is>
+          <t>Mokosh</t>
+        </is>
+      </c>
+      <c r="B37" s="2" t="inlineStr">
+        <is>
+          <t>https://mokosh.pl/</t>
+        </is>
+      </c>
+      <c r="C37" s="2" t="inlineStr">
+        <is>
+          <t>Poland</t>
+        </is>
+      </c>
+      <c r="D37" s="3" t="inlineStr">
+        <is>
+          <t>https://mokosh.pl/policies/terms-of-service — 'MOKOSH Didiuk sp. k. z siedzibą: ul. Dolna 14, 05-152 Kazuń Nowy'</t>
+        </is>
+      </c>
+      <c r="E37" s="2" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="F37" s="2" t="inlineStr">
+        <is>
+          <t>Beauty / natural cosmetics</t>
+        </is>
+      </c>
+      <c r="G37" s="3" t="inlineStr">
+        <is>
+          <t>Bronzing body &amp; face balm, orange with cinnamon</t>
+        </is>
+      </c>
+      <c r="H37" s="2" t="inlineStr">
+        <is>
+          <t>89 zł</t>
+        </is>
+      </c>
+      <c r="I37" s="2" t="inlineStr">
+        <is>
+          <t>biuro@mokosh.pl</t>
+        </is>
+      </c>
+      <c r="J37" s="2" t="inlineStr"/>
+      <c r="K37" s="3" t="inlineStr">
+        <is>
+          <t>none on site; TikTok profile not a seller account</t>
+        </is>
+      </c>
+      <c r="L37" s="2" t="inlineStr"/>
+      <c r="M37" s="3" t="inlineStr"/>
+      <c r="N37" s="3" t="inlineStr">
+        <is>
+          <t>Site lists Hungary (Węgry) among countries where Mokosh sells</t>
+        </is>
+      </c>
+      <c r="O37" s="3" t="inlineStr">
+        <is>
+          <t>Your bronzing body and face balm with orange and cinnamon is exactly the kind of product that sells on TikTok: the glow is visible before and after in one short video.</t>
+        </is>
+      </c>
+      <c r="P37" s="2" t="inlineStr">
+        <is>
+          <t>beauty and skincare creators</t>
+        </is>
+      </c>
+      <c r="Q37" s="3" t="inlineStr"/>
+      <c r="R37" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-26</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="2" t="inlineStr">
+        <is>
+          <t>Sylveco</t>
+        </is>
+      </c>
+      <c r="B38" s="2" t="inlineStr">
+        <is>
+          <t>https://sylveco.pl/</t>
+        </is>
+      </c>
+      <c r="C38" s="2" t="inlineStr">
+        <is>
+          <t>Poland</t>
+        </is>
+      </c>
+      <c r="D38" s="3" t="inlineStr">
+        <is>
+          <t>https://sylveco.pl/regulamin/ — 'SYLVECO spółka z o.o. … z siedzibą w 36-004 Łąka k/Rzeszowa'</t>
+        </is>
+      </c>
+      <c r="E38" s="2" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="F38" s="2" t="inlineStr">
+        <is>
+          <t>Beauty / natural skincare</t>
+        </is>
+      </c>
+      <c r="G38" s="3" t="inlineStr">
+        <is>
+          <t>SYLVECO birch cream with betulin (Krem brzozowy z betuliną) 50ml</t>
+        </is>
+      </c>
+      <c r="H38" s="2" t="inlineStr">
+        <is>
+          <t>53,99 zł</t>
+        </is>
+      </c>
+      <c r="I38" s="2" t="inlineStr">
+        <is>
+          <t>export@sylveco.pl</t>
+        </is>
+      </c>
+      <c r="J38" s="2" t="inlineStr"/>
+      <c r="K38" s="3" t="inlineStr">
+        <is>
+          <t>none on site; @sylveco.pl is not a TikTok Shop seller account</t>
+        </is>
+      </c>
+      <c r="L38" s="2" t="inlineStr"/>
+      <c r="M38" s="3" t="inlineStr"/>
+      <c r="N38" s="3" t="inlineStr">
+        <is>
+          <t>Ships to Hungary: shipping price list on sylveco.pl includes 'Węgry'</t>
+        </is>
+      </c>
+      <c r="O38" s="3" t="inlineStr">
+        <is>
+          <t>Your birch cream with betulin, one of your bestsellers, is a simple product to show in a short skincare video, with a natural-ingredient story creators can explain in seconds.</t>
+        </is>
+      </c>
+      <c r="P38" s="2" t="inlineStr">
+        <is>
+          <t>beauty and skincare creators</t>
+        </is>
+      </c>
+      <c r="Q38" s="3" t="inlineStr"/>
+      <c r="R38" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-26</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="2" t="inlineStr">
+        <is>
+          <t>Emma Hardie</t>
+        </is>
+      </c>
+      <c r="B39" s="2" t="inlineStr">
+        <is>
+          <t>https://shop.emmahardie.com/</t>
+        </is>
+      </c>
+      <c r="C39" s="2" t="inlineStr">
+        <is>
+          <t>United Kingdom</t>
+        </is>
+      </c>
+      <c r="D39" s="3" t="inlineStr">
+        <is>
+          <t>https://shop.emmahardie.com/pages/terms-of-use — 'registered address is 2nd Floor, 66-68 Margaret Street London W1W 8SR'</t>
+        </is>
+      </c>
+      <c r="E39" s="2" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="F39" s="2" t="inlineStr">
+        <is>
+          <t>Beauty / skincare</t>
+        </is>
+      </c>
+      <c r="G39" s="3" t="inlineStr">
+        <is>
+          <t>Moringa Cleansing Balm with Dual Action Cleansing Cloth</t>
+        </is>
+      </c>
+      <c r="H39" s="2" t="inlineStr">
+        <is>
+          <t>£52</t>
+        </is>
+      </c>
+      <c r="I39" s="2" t="inlineStr">
+        <is>
+          <t>info@emmahardie.com</t>
+        </is>
+      </c>
+      <c r="J39" s="2" t="inlineStr"/>
+      <c r="K39" s="3" t="inlineStr">
+        <is>
+          <t>none on site; @emmahardie is not a TikTok Shop seller account</t>
+        </is>
+      </c>
+      <c r="L39" s="2" t="inlineStr"/>
+      <c r="M39" s="3" t="inlineStr"/>
+      <c r="N39" s="3" t="inlineStr">
+        <is>
+          <t>Ships to Hungary: Hungary (HUF Ft) in the site's country/currency selector</t>
+        </is>
+      </c>
+      <c r="O39" s="3" t="inlineStr">
+        <is>
+          <t>Your Moringa Cleansing Balm with Dual Action Cleansing Cloth is easy to demonstrate on camera: makeup on, balm and cloth, makeup off, all in one short video.</t>
+        </is>
+      </c>
+      <c r="P39" s="2" t="inlineStr">
+        <is>
+          <t>beauty and skincare creators</t>
+        </is>
+      </c>
+      <c r="Q39" s="3" t="inlineStr"/>
+      <c r="R39" s="2" t="inlineStr">
         <is>
           <t>2026-09-26</t>
         </is>

</xml_diff>

<commit_message>
Contact email priority (marketing/partnerships/PR/affiliate first) and apply to batch 2026-09-28
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_015V3tpdvHrRGbX5pxPwM4Y2
</commit_message>
<xml_diff>
--- a/brands_intl.xlsx
+++ b/brands_intl.xlsx
@@ -434,7 +434,7 @@
     <col width="28" customWidth="1" min="6" max="6"/>
     <col width="60" customWidth="1" min="7" max="7"/>
     <col width="18" customWidth="1" min="8" max="8"/>
-    <col width="36" customWidth="1" min="9" max="9"/>
+    <col width="35" customWidth="1" min="9" max="9"/>
     <col width="12" customWidth="1" min="10" max="10"/>
     <col width="60" customWidth="1" min="11" max="11"/>
     <col width="27" customWidth="1" min="12" max="12"/>
@@ -1469,7 +1469,7 @@
       </c>
       <c r="I13" s="2" t="inlineStr">
         <is>
-          <t>hello@beautykitchen.co.uk</t>
+          <t>pr@beautykitchen.co.uk</t>
         </is>
       </c>
       <c r="J13" s="2" t="inlineStr"/>
@@ -1629,7 +1629,7 @@
       </c>
       <c r="I15" s="2" t="inlineStr">
         <is>
-          <t>wecare@betteryou.com</t>
+          <t>media@betteryou.com</t>
         </is>
       </c>
       <c r="J15" s="2" t="inlineStr"/>
@@ -1709,7 +1709,7 @@
       </c>
       <c r="I16" s="2" t="inlineStr">
         <is>
-          <t>customercare@bperfectcosmetics.com</t>
+          <t>aff@bperfectcosmetics.com</t>
         </is>
       </c>
       <c r="J16" s="2" t="inlineStr"/>
@@ -2353,7 +2353,7 @@
       </c>
       <c r="I24" s="2" t="inlineStr">
         <is>
-          <t>hello@nailsinc.com</t>
+          <t>press@nailsinc.com</t>
         </is>
       </c>
       <c r="J24" s="2" t="inlineStr"/>
@@ -2673,7 +2673,7 @@
       </c>
       <c r="I28" s="2" t="inlineStr">
         <is>
-          <t>info@orelia.co.uk</t>
+          <t>press@orelia.co.uk</t>
         </is>
       </c>
       <c r="J28" s="2" t="inlineStr"/>

</xml_diff>

<commit_message>
Auto-reply/stop handling, contacts lookup, greetings from named contacts, new creators
- mark --auto-reply (recorded, not a reply) and --stop (ends follow-ups); Hairburst support@ stopped
- pipeline/contacts.py: founder / head of marketing / e-commerce manager from brand sites and
  LinkedIn search results -> linkedin_contacts.xlsx; greeting uses the name when found
- creators.csv: Laura (@lauritaabotos), Noémi (@tothnoemiiii)
- send refuses to run before a batch's scheduled date
- Batch 2026-09-28 rebuilt with named greetings and re-approved

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_015V3tpdvHrRGbX5pxPwM4Y2
</commit_message>
<xml_diff>
--- a/brands_intl.xlsx
+++ b/brands_intl.xlsx
@@ -435,7 +435,7 @@
     <col width="60" customWidth="1" min="7" max="7"/>
     <col width="18" customWidth="1" min="8" max="8"/>
     <col width="35" customWidth="1" min="9" max="9"/>
-    <col width="12" customWidth="1" min="10" max="10"/>
+    <col width="15" customWidth="1" min="10" max="10"/>
     <col width="60" customWidth="1" min="11" max="11"/>
     <col width="27" customWidth="1" min="12" max="12"/>
     <col width="60" customWidth="1" min="13" max="13"/>
@@ -908,7 +908,11 @@
           <t>hello@boskanails.pl</t>
         </is>
       </c>
-      <c r="J6" s="2" t="inlineStr"/>
+      <c r="J6" s="2" t="inlineStr">
+        <is>
+          <t>Maciej</t>
+        </is>
+      </c>
       <c r="K6" s="3" t="inlineStr">
         <is>
           <t>TikTok profile @boskanailspl is a TikTok Shop seller account (ttSeller)</t>
@@ -1712,7 +1716,11 @@
           <t>aff@bperfectcosmetics.com</t>
         </is>
       </c>
-      <c r="J16" s="2" t="inlineStr"/>
+      <c r="J16" s="2" t="inlineStr">
+        <is>
+          <t>Brendan</t>
+        </is>
+      </c>
       <c r="K16" s="3" t="inlineStr">
         <is>
           <t>About page: 'one of the Top 3 UK brands on TikTok Shop'; TikTok profile @bperfectcosmetics is a TikTok Shop seller account (ttSeller)</t>
@@ -2356,7 +2364,11 @@
           <t>press@nailsinc.com</t>
         </is>
       </c>
-      <c r="J24" s="2" t="inlineStr"/>
+      <c r="J24" s="2" t="inlineStr">
+        <is>
+          <t>Thea</t>
+        </is>
+      </c>
       <c r="K24" s="3" t="inlineStr">
         <is>
           <t>TikTok profile @nailsinclondon is a TikTok Shop seller account (ttSeller)</t>
@@ -2516,7 +2528,11 @@
           <t>enquiries@nipandfab.com</t>
         </is>
       </c>
-      <c r="J26" s="2" t="inlineStr"/>
+      <c r="J26" s="2" t="inlineStr">
+        <is>
+          <t>Maria</t>
+        </is>
+      </c>
       <c r="K26" s="3" t="inlineStr">
         <is>
           <t>TikTok profile @nipandfab is a TikTok Shop seller account (ttSeller)</t>
@@ -2676,7 +2692,11 @@
           <t>press@orelia.co.uk</t>
         </is>
       </c>
-      <c r="J28" s="2" t="inlineStr"/>
+      <c r="J28" s="2" t="inlineStr">
+        <is>
+          <t>Collette</t>
+        </is>
+      </c>
       <c r="K28" s="3" t="inlineStr">
         <is>
           <t>TikTok profile @oreliajewellery is a TikTok Shop seller account (ttSeller)</t>
@@ -3076,7 +3096,11 @@
           <t>hello@upcirclebeauty.com</t>
         </is>
       </c>
-      <c r="J33" s="2" t="inlineStr"/>
+      <c r="J33" s="2" t="inlineStr">
+        <is>
+          <t>Will and Anna</t>
+        </is>
+      </c>
       <c r="K33" s="3" t="inlineStr">
         <is>
           <t>TikTok profile @upcirclebeauty is a TikTok Shop seller account (ttSeller)</t>
@@ -3304,7 +3328,11 @@
           <t>info@makear.pl</t>
         </is>
       </c>
-      <c r="J36" s="2" t="inlineStr"/>
+      <c r="J36" s="2" t="inlineStr">
+        <is>
+          <t>Robert</t>
+        </is>
+      </c>
       <c r="K36" s="3" t="inlineStr">
         <is>
           <t>none on site; @makear is not a TikTok Shop seller account</t>

</xml_diff>